<commit_message>
Update binary files and enhance stringing and erection data handling
- Updated multiple binary files including `ErectionCompiled_Output.xlsx`, `MicroPlanIndex.parquet`, and `StringingCompiled_Output.xlsx` to reflect recent changes in data processing.
- Deleted outdated DPR Excel files to clean up the project directory.
- Improved callback logic in `dashboard/callbacks.py` for better data retrieval and processing.
- Enhanced functions for managing stringing plan data and project filtering capabilities.
</commit_message>
<xml_diff>
--- a/Raw Data/Micro Plans/November 2025/Micro Plan - TA-421 Nov'25.xlsx
+++ b/Raw Data/Micro Plans/November 2025/Micro Plan - TA-421 Nov'25.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kaushikb\Documents\Work\Git\Office-work-\Raw Data\Micro Plans\November 2025\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0ABE5E5B-1032-43D4-BF9B-84C78188882A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C965881B-D56B-4EDF-9D96-6A23D224259C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="757" firstSheet="2" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1777,96 +1777,6 @@
     <xf numFmtId="14" fontId="31" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="33" fillId="2" borderId="15" xfId="27" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1911,6 +1821,96 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="20" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -2022,6 +2022,16 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF006100"/>
       </font>
       <fill>
@@ -2042,6 +2052,26 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
@@ -2062,6 +2092,26 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF9C5700"/>
       </font>
       <fill>
@@ -2072,6 +2122,16 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF006100"/>
       </font>
       <fill>
@@ -2102,6 +2162,16 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
@@ -2112,6 +2182,16 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF9C5700"/>
       </font>
       <fill>
@@ -2142,6 +2222,26 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF006100"/>
       </font>
       <fill>
@@ -2152,6 +2252,46 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF9C5700"/>
       </font>
       <fill>
@@ -2162,6 +2302,16 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
@@ -2182,6 +2332,46 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF9C5700"/>
       </font>
       <fill>
@@ -2202,6 +2392,16 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
@@ -2252,6 +2452,16 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF006100"/>
       </font>
       <fill>
@@ -2262,6 +2472,16 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
@@ -2272,6 +2492,16 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
@@ -2292,261 +2522,31 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF9C5700"/>
       </font>
       <fill>
         <patternFill>
           <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2892,6 +2892,31 @@
     </dxf>
     <dxf>
       <font>
+        <color indexed="20"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor indexed="45"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color indexed="20"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor indexed="45"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color indexed="20"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
         <color indexed="17"/>
       </font>
       <fill>
@@ -2899,31 +2924,6 @@
           <bgColor indexed="42"/>
         </patternFill>
       </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color indexed="20"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor indexed="45"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color indexed="20"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor indexed="45"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color indexed="20"/>
-      </font>
     </dxf>
     <dxf>
       <font>
@@ -3745,137 +3745,137 @@
       <c r="F17" s="6"/>
     </row>
     <row r="18" spans="1:33" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="179" t="s">
+      <c r="A18" s="180" t="s">
         <v>4</v>
       </c>
-      <c r="B18" s="179" t="s">
+      <c r="B18" s="180" t="s">
         <v>5</v>
       </c>
-      <c r="C18" s="175" t="s">
+      <c r="C18" s="177" t="s">
         <v>6</v>
       </c>
-      <c r="D18" s="179" t="s">
+      <c r="D18" s="180" t="s">
         <v>7</v>
       </c>
-      <c r="E18" s="175" t="s">
+      <c r="E18" s="177" t="s">
         <v>16</v>
       </c>
-      <c r="F18" s="175" t="s">
+      <c r="F18" s="177" t="s">
         <v>17</v>
       </c>
-      <c r="G18" s="179" t="s">
+      <c r="G18" s="180" t="s">
         <v>8</v>
       </c>
-      <c r="H18" s="166" t="s">
+      <c r="H18" s="192" t="s">
         <v>18</v>
       </c>
-      <c r="I18" s="166"/>
-      <c r="J18" s="166"/>
-      <c r="K18" s="166"/>
-      <c r="L18" s="166"/>
-      <c r="M18" s="166"/>
-      <c r="N18" s="166"/>
-      <c r="O18" s="166"/>
-      <c r="P18" s="169" t="s">
+      <c r="I18" s="192"/>
+      <c r="J18" s="192"/>
+      <c r="K18" s="192"/>
+      <c r="L18" s="192"/>
+      <c r="M18" s="192"/>
+      <c r="N18" s="192"/>
+      <c r="O18" s="192"/>
+      <c r="P18" s="185" t="s">
         <v>19</v>
       </c>
-      <c r="R18" s="175" t="s">
+      <c r="R18" s="177" t="s">
         <v>36</v>
       </c>
-      <c r="T18" s="170" t="s">
+      <c r="T18" s="186" t="s">
         <v>31</v>
       </c>
-      <c r="U18" s="171"/>
-      <c r="V18" s="171"/>
-      <c r="W18" s="171"/>
-      <c r="X18" s="171"/>
-      <c r="Y18" s="172"/>
-      <c r="AA18" s="170" t="s">
+      <c r="U18" s="187"/>
+      <c r="V18" s="187"/>
+      <c r="W18" s="187"/>
+      <c r="X18" s="187"/>
+      <c r="Y18" s="188"/>
+      <c r="AA18" s="186" t="s">
         <v>30</v>
       </c>
-      <c r="AB18" s="171"/>
-      <c r="AC18" s="171"/>
-      <c r="AD18" s="171"/>
-      <c r="AE18" s="171"/>
-      <c r="AF18" s="172"/>
-      <c r="AG18" s="173" t="s">
+      <c r="AB18" s="187"/>
+      <c r="AC18" s="187"/>
+      <c r="AD18" s="187"/>
+      <c r="AE18" s="187"/>
+      <c r="AF18" s="188"/>
+      <c r="AG18" s="189" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="19" spans="1:33" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="180"/>
-      <c r="B19" s="180"/>
-      <c r="C19" s="177"/>
-      <c r="D19" s="180"/>
-      <c r="E19" s="177"/>
-      <c r="F19" s="177"/>
-      <c r="G19" s="180"/>
-      <c r="H19" s="165" t="s">
+      <c r="A19" s="181"/>
+      <c r="B19" s="181"/>
+      <c r="C19" s="178"/>
+      <c r="D19" s="181"/>
+      <c r="E19" s="178"/>
+      <c r="F19" s="178"/>
+      <c r="G19" s="181"/>
+      <c r="H19" s="197" t="s">
         <v>9</v>
       </c>
-      <c r="I19" s="165"/>
-      <c r="J19" s="165" t="s">
+      <c r="I19" s="197"/>
+      <c r="J19" s="197" t="s">
         <v>12</v>
       </c>
-      <c r="K19" s="165"/>
-      <c r="L19" s="165" t="s">
+      <c r="K19" s="197"/>
+      <c r="L19" s="197" t="s">
         <v>13</v>
       </c>
-      <c r="M19" s="165"/>
-      <c r="N19" s="163" t="s">
+      <c r="M19" s="197"/>
+      <c r="N19" s="193" t="s">
         <v>15</v>
       </c>
-      <c r="O19" s="163" t="s">
+      <c r="O19" s="193" t="s">
         <v>14</v>
       </c>
-      <c r="P19" s="169"/>
-      <c r="R19" s="176"/>
-      <c r="T19" s="167" t="s">
+      <c r="P19" s="185"/>
+      <c r="R19" s="191"/>
+      <c r="T19" s="183" t="s">
         <v>24</v>
       </c>
-      <c r="U19" s="167" t="s">
+      <c r="U19" s="183" t="s">
         <v>25</v>
       </c>
-      <c r="V19" s="167" t="s">
+      <c r="V19" s="183" t="s">
         <v>26</v>
       </c>
-      <c r="W19" s="167" t="s">
+      <c r="W19" s="183" t="s">
         <v>27</v>
       </c>
-      <c r="X19" s="167" t="s">
+      <c r="X19" s="183" t="s">
         <v>28</v>
       </c>
       <c r="Y19" s="43" t="s">
         <v>29</v>
       </c>
-      <c r="AA19" s="167" t="s">
+      <c r="AA19" s="183" t="s">
         <v>24</v>
       </c>
-      <c r="AB19" s="167" t="s">
+      <c r="AB19" s="183" t="s">
         <v>25</v>
       </c>
-      <c r="AC19" s="167" t="s">
+      <c r="AC19" s="183" t="s">
         <v>26</v>
       </c>
-      <c r="AD19" s="167" t="s">
+      <c r="AD19" s="183" t="s">
         <v>27</v>
       </c>
-      <c r="AE19" s="167" t="s">
+      <c r="AE19" s="183" t="s">
         <v>28</v>
       </c>
       <c r="AF19" s="43" t="s">
         <v>29</v>
       </c>
-      <c r="AG19" s="174"/>
+      <c r="AG19" s="190"/>
     </row>
     <row r="20" spans="1:33" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A20" s="181"/>
-      <c r="B20" s="180"/>
-      <c r="C20" s="177"/>
-      <c r="D20" s="180"/>
-      <c r="E20" s="178"/>
-      <c r="F20" s="178"/>
-      <c r="G20" s="180"/>
+      <c r="A20" s="182"/>
+      <c r="B20" s="181"/>
+      <c r="C20" s="178"/>
+      <c r="D20" s="181"/>
+      <c r="E20" s="179"/>
+      <c r="F20" s="179"/>
+      <c r="G20" s="181"/>
       <c r="H20" s="94" t="s">
         <v>10</v>
       </c>
@@ -3894,25 +3894,25 @@
       <c r="M20" s="94" t="s">
         <v>11</v>
       </c>
-      <c r="N20" s="164"/>
-      <c r="O20" s="164"/>
+      <c r="N20" s="194"/>
+      <c r="O20" s="194"/>
       <c r="P20" s="44" t="s">
         <v>50</v>
       </c>
       <c r="R20" s="18" t="s">
         <v>37</v>
       </c>
-      <c r="T20" s="168"/>
-      <c r="U20" s="168"/>
-      <c r="V20" s="168"/>
-      <c r="W20" s="168"/>
-      <c r="X20" s="168"/>
+      <c r="T20" s="184"/>
+      <c r="U20" s="184"/>
+      <c r="V20" s="184"/>
+      <c r="W20" s="184"/>
+      <c r="X20" s="184"/>
       <c r="Y20" s="19"/>
-      <c r="AA20" s="168"/>
-      <c r="AB20" s="168"/>
-      <c r="AC20" s="168"/>
-      <c r="AD20" s="168"/>
-      <c r="AE20" s="168"/>
+      <c r="AA20" s="184"/>
+      <c r="AB20" s="184"/>
+      <c r="AC20" s="184"/>
+      <c r="AD20" s="184"/>
+      <c r="AE20" s="184"/>
       <c r="AF20" s="19" t="s">
         <v>50</v>
       </c>
@@ -4183,7 +4183,7 @@
       <c r="D25" s="86"/>
       <c r="E25" s="101"/>
       <c r="F25" s="8"/>
-      <c r="G25" s="161"/>
+      <c r="G25" s="195"/>
       <c r="H25" s="99"/>
       <c r="I25" s="99"/>
       <c r="J25" s="99"/>
@@ -4241,7 +4241,7 @@
       <c r="D26" s="8"/>
       <c r="E26" s="102"/>
       <c r="F26" s="97"/>
-      <c r="G26" s="162"/>
+      <c r="G26" s="196"/>
       <c r="H26" s="99"/>
       <c r="I26" s="99"/>
       <c r="J26" s="99"/>
@@ -4596,13 +4596,16 @@
     <filterColumn colId="13" showButton="0"/>
   </autoFilter>
   <mergeCells count="29">
-    <mergeCell ref="F18:F20"/>
-    <mergeCell ref="G18:G20"/>
-    <mergeCell ref="A18:A20"/>
-    <mergeCell ref="B18:B20"/>
-    <mergeCell ref="C18:C20"/>
-    <mergeCell ref="D18:D20"/>
-    <mergeCell ref="E18:E20"/>
+    <mergeCell ref="G25:G26"/>
+    <mergeCell ref="O19:O20"/>
+    <mergeCell ref="H19:I19"/>
+    <mergeCell ref="J19:K19"/>
+    <mergeCell ref="L19:M19"/>
+    <mergeCell ref="H18:O18"/>
+    <mergeCell ref="N19:N20"/>
+    <mergeCell ref="U19:U20"/>
+    <mergeCell ref="V19:V20"/>
+    <mergeCell ref="W19:W20"/>
     <mergeCell ref="X19:X20"/>
     <mergeCell ref="P18:P19"/>
     <mergeCell ref="AA18:AF18"/>
@@ -4615,16 +4618,13 @@
     <mergeCell ref="R18:R19"/>
     <mergeCell ref="T18:Y18"/>
     <mergeCell ref="T19:T20"/>
-    <mergeCell ref="H18:O18"/>
-    <mergeCell ref="N19:N20"/>
-    <mergeCell ref="U19:U20"/>
-    <mergeCell ref="V19:V20"/>
-    <mergeCell ref="W19:W20"/>
-    <mergeCell ref="G25:G26"/>
-    <mergeCell ref="O19:O20"/>
-    <mergeCell ref="H19:I19"/>
-    <mergeCell ref="J19:K19"/>
-    <mergeCell ref="L19:M19"/>
+    <mergeCell ref="F18:F20"/>
+    <mergeCell ref="G18:G20"/>
+    <mergeCell ref="A18:A20"/>
+    <mergeCell ref="B18:B20"/>
+    <mergeCell ref="C18:C20"/>
+    <mergeCell ref="D18:D20"/>
+    <mergeCell ref="E18:E20"/>
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B21">
@@ -4699,17 +4699,17 @@
     <cfRule type="expression" dxfId="99" priority="1243" stopIfTrue="1">
       <formula>AND(COUNTIF($D$1:$D$123, B26)+COUNTIF($D$142:$D$65380, B26)&gt;1,NOT(ISBLANK(B26)))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="98" priority="1245" stopIfTrue="1">
+    <cfRule type="expression" dxfId="98" priority="1244" stopIfTrue="1">
       <formula>AND(COUNTIF($D$1:$D$191, B26)+COUNTIF($D$214:$D$65380, B26)&gt;1,NOT(ISBLANK(B26)))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="97" priority="1246" stopIfTrue="1">
+    <cfRule type="expression" dxfId="97" priority="1245" stopIfTrue="1">
       <formula>AND(COUNTIF($D$1:$D$191, B26)+COUNTIF($D$214:$D$65380, B26)&gt;1,NOT(ISBLANK(B26)))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="96" priority="1247" stopIfTrue="1">
+    <cfRule type="expression" dxfId="96" priority="1246" stopIfTrue="1">
+      <formula>AND(COUNTIF($D$1:$D$191, B26)+COUNTIF($D$214:$D$65380, B26)&gt;1,NOT(ISBLANK(B26)))</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="95" priority="1247" stopIfTrue="1">
       <formula>AND(COUNTIF($D$474:$D$65380, B26)+COUNTIF($D$454:$D$455, B26)+COUNTIF($D$416:$D$417, B26)+COUNTIF($D$374:$D$377, B26)+COUNTIF($D$351:$D$352, B26)+COUNTIF($D$324:$D$325, B26)+COUNTIF($D$303:$D$303, B26)+COUNTIF($D$288:$D$289, B26)+COUNTIF($D$263:$D$263, B26)+COUNTIF($D$252:$D$253, B26)+COUNTIF($D$233:$D$234, B26)+COUNTIF($D$51:$D$218, B26)+COUNTIF($D$219:$D$220, B26)+COUNTIF($D$1:$D$50, B26)&gt;1,NOT(ISBLANK(B26)))</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="95" priority="1244" stopIfTrue="1">
-      <formula>AND(COUNTIF($D$1:$D$191, B26)+COUNTIF($D$214:$D$65380, B26)&gt;1,NOT(ISBLANK(B26)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B27">
@@ -4726,55 +4726,55 @@
     <cfRule type="duplicateValues" dxfId="88" priority="347"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="L4">
-    <cfRule type="expression" dxfId="87" priority="1221" stopIfTrue="1">
+    <cfRule type="expression" dxfId="87" priority="1220" stopIfTrue="1">
+      <formula>AND(COUNTIF($C$314:$C$65460, L4)+COUNTIF($C$294:$C$295, L4)+COUNTIF($C$256:$C$257, L4)+COUNTIF($C$214:$C$217, L4)+COUNTIF($C$191:$C$192, L4)+COUNTIF($C$164:$C$165, L4)+COUNTIF($C$143:$C$143, L4)+COUNTIF($C$128:$C$129, L4)+COUNTIF($C$103:$C$103, L4)+COUNTIF($C$92:$C$93, L4)+COUNTIF($C$73:$C$74, L4)+COUNTIF($C$29:$C$56, L4)+COUNTIF($C$58:$C$60, L4)+COUNTIF($C$1:$C$27, L4)&gt;1,NOT(ISBLANK(L4)))</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="86" priority="1221" stopIfTrue="1">
       <formula>AND(COUNTIF($C$1:$C$65460, L4)+COUNTIF(#REF!, L4)&gt;1,NOT(ISBLANK(L4)))</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="86" priority="1220" stopIfTrue="1">
-      <formula>AND(COUNTIF($C$314:$C$65460, L4)+COUNTIF($C$294:$C$295, L4)+COUNTIF($C$256:$C$257, L4)+COUNTIF($C$214:$C$217, L4)+COUNTIF($C$191:$C$192, L4)+COUNTIF($C$164:$C$165, L4)+COUNTIF($C$143:$C$143, L4)+COUNTIF($C$128:$C$129, L4)+COUNTIF($C$103:$C$103, L4)+COUNTIF($C$92:$C$93, L4)+COUNTIF($C$73:$C$74, L4)+COUNTIF($C$29:$C$56, L4)+COUNTIF($C$58:$C$60, L4)+COUNTIF($C$1:$C$27, L4)&gt;1,NOT(ISBLANK(L4)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M4">
-    <cfRule type="expression" dxfId="85" priority="1223" stopIfTrue="1">
+    <cfRule type="expression" dxfId="85" priority="1222" stopIfTrue="1">
+      <formula>AND(COUNTIF($D$331:$D$65460, M4)+COUNTIF($D$1:$D$27, M4)+COUNTIF(#REF!, M4)+COUNTIF($D$314:$D$315, M4)+COUNTIF($D$294:$D$295, M4)+COUNTIF($D$256:$D$257, M4)+COUNTIF($D$214:$D$217, M4)+COUNTIF($D$191:$D$192, M4)+COUNTIF($D$164:$D$165, M4)+COUNTIF($D$143:$D$143, M4)+COUNTIF($D$128:$D$129, M4)+COUNTIF($D$103:$D$103, M4)+COUNTIF($D$92:$D$93, M4)+COUNTIF($D$73:$D$74, M4)+COUNTIF($D$58:$D$60, M4)&gt;1,NOT(ISBLANK(M4)))</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="84" priority="1223" stopIfTrue="1">
       <formula>AND(COUNTIF($D$314:$D$65460, M4)+COUNTIF(#REF!, M4)+COUNTIF($D$1:$D$27, M4)+COUNTIF($D$294:$D$295, M4)+COUNTIF($D$256:$D$257, M4)+COUNTIF($D$214:$D$217, M4)+COUNTIF($D$191:$D$192, M4)+COUNTIF($D$164:$D$165, M4)+COUNTIF($D$143:$D$143, M4)+COUNTIF($D$128:$D$129, M4)+COUNTIF($D$103:$D$103, M4)+COUNTIF($D$92:$D$93, M4)+COUNTIF($D$73:$D$74, M4)+COUNTIF($D$58:$D$60, M4)&gt;1,NOT(ISBLANK(M4)))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="84" priority="1224" stopIfTrue="1">
+    <cfRule type="expression" dxfId="83" priority="1224" stopIfTrue="1">
       <formula>AND(COUNTIF($D$294:$D$65460, M4)+COUNTIF($D$1:$D$27, M4)+COUNTIF($D$256:$D$257, M4)+COUNTIF(#REF!, M4)+COUNTIF($D$214:$D$217, M4)+COUNTIF($D$191:$D$192, M4)+COUNTIF($D$164:$D$165, M4)+COUNTIF($D$143:$D$143, M4)+COUNTIF($D$128:$D$129, M4)+COUNTIF($D$103:$D$103, M4)+COUNTIF($D$92:$D$93, M4)+COUNTIF($D$73:$D$74, M4)+COUNTIF($D$58:$D$60, M4)&gt;1,NOT(ISBLANK(M4)))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="83" priority="1225" stopIfTrue="1">
+    <cfRule type="expression" dxfId="82" priority="1225" stopIfTrue="1">
       <formula>AND(COUNTIF($D$256:$D$65460, M4)+COUNTIF($D$1:$D$27, M4)+COUNTIF(#REF!, M4)+COUNTIF($D$214:$D$217, M4)+COUNTIF($D$191:$D$192, M4)+COUNTIF($D$164:$D$165, M4)+COUNTIF($D$143:$D$143, M4)+COUNTIF($D$128:$D$129, M4)+COUNTIF($D$103:$D$103, M4)+COUNTIF($D$92:$D$93, M4)+COUNTIF($D$73:$D$74, M4)+COUNTIF($D$58:$D$60, M4)&gt;1,NOT(ISBLANK(M4)))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="82" priority="1226" stopIfTrue="1">
+    <cfRule type="expression" dxfId="81" priority="1226" stopIfTrue="1">
       <formula>AND(COUNTIF($D$214:$D$65460, M4)+COUNTIF(#REF!, M4)+COUNTIF($D$1:$D$27, M4)+COUNTIF($D$191:$D$192, M4)+COUNTIF($D$164:$D$165, M4)+COUNTIF($D$143:$D$143, M4)+COUNTIF($D$128:$D$129, M4)+COUNTIF($D$103:$D$103, M4)+COUNTIF($D$92:$D$93, M4)+COUNTIF($D$73:$D$74, M4)+COUNTIF($D$58:$D$60, M4)&gt;1,NOT(ISBLANK(M4)))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="81" priority="1227" stopIfTrue="1">
+    <cfRule type="expression" dxfId="80" priority="1227" stopIfTrue="1">
       <formula>AND(COUNTIF($D$214:$D$65460, M4)+COUNTIF($D$191:$D$192, M4)+COUNTIF($D$164:$D$165, M4)+COUNTIF($D$143:$D$143, M4)+COUNTIF($D$128:$D$129, M4)+COUNTIF($D$1:$D$27, M4)+COUNTIF(#REF!, M4)+COUNTIF($D$103:$D$103, M4)+COUNTIF($D$92:$D$93, M4)+COUNTIF(#REF!, M4)+COUNTIF($D$73:$D$74, M4)+COUNTIF($D$51:$D$51, M4)+COUNTIF($D$53:$D$60, M4)+COUNTIF(#REF!, M4)&gt;1,NOT(ISBLANK(M4)))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="80" priority="1228" stopIfTrue="1">
+    <cfRule type="expression" dxfId="79" priority="1228" stopIfTrue="1">
       <formula>AND(COUNTIF($D$191:$D$65460, M4)+COUNTIF($D$164:$D$165, M4)+COUNTIF($D$143:$D$143, M4)+COUNTIF($D$128:$D$129, M4)+COUNTIF($D$1:$D$27, M4)+COUNTIF(#REF!, M4)+COUNTIF($D$103:$D$103, M4)+COUNTIF($D$92:$D$93, M4)+COUNTIF(#REF!, M4)+COUNTIF($D$73:$D$74, M4)+COUNTIF($D$51:$D$51, M4)+COUNTIF($D$53:$D$60, M4)+COUNTIF(#REF!, M4)&gt;1,NOT(ISBLANK(M4)))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="79" priority="1229" stopIfTrue="1">
+    <cfRule type="expression" dxfId="78" priority="1229" stopIfTrue="1">
       <formula>AND(COUNTIF($F$369:$F$65454, M4)+COUNTIF($F$1:$F$27, M4)+COUNTIF(#REF!, M4)+COUNTIF($F$352:$F$353, M4)+COUNTIF($F$332:$F$333, M4)+COUNTIF($F$294:$F$295, M4)+COUNTIF($F$252:$F$255, M4)+COUNTIF($F$229:$F$230, M4)+COUNTIF($F$202:$F$203, M4)+COUNTIF($F$181:$F$181, M4)+COUNTIF($F$166:$F$167, M4)+COUNTIF($F$141:$F$141, M4)+COUNTIF($F$130:$F$131, M4)+COUNTIF($F$111:$F$112, M4)+COUNTIF($F$96:$F$98, M4)&gt;1,NOT(ISBLANK(M4)))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="78" priority="1230" stopIfTrue="1">
+    <cfRule type="expression" dxfId="77" priority="1230" stopIfTrue="1">
       <formula>AND(COUNTIF($F$352:$F$65454, M4)+COUNTIF(#REF!, M4)+COUNTIF($F$1:$F$27, M4)+COUNTIF($F$332:$F$333, M4)+COUNTIF($F$294:$F$295, M4)+COUNTIF($F$252:$F$255, M4)+COUNTIF($F$229:$F$230, M4)+COUNTIF($F$202:$F$203, M4)+COUNTIF($F$181:$F$181, M4)+COUNTIF($F$166:$F$167, M4)+COUNTIF($F$141:$F$141, M4)+COUNTIF($F$130:$F$131, M4)+COUNTIF($F$111:$F$112, M4)+COUNTIF($F$96:$F$98, M4)&gt;1,NOT(ISBLANK(M4)))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="77" priority="1231" stopIfTrue="1">
+    <cfRule type="expression" dxfId="76" priority="1231" stopIfTrue="1">
       <formula>AND(COUNTIF($F$332:$F$65454, M4)+COUNTIF($F$1:$F$27, M4)+COUNTIF($F$294:$F$295, M4)+COUNTIF(#REF!, M4)+COUNTIF($F$252:$F$255, M4)+COUNTIF($F$229:$F$230, M4)+COUNTIF($F$202:$F$203, M4)+COUNTIF($F$181:$F$181, M4)+COUNTIF($F$166:$F$167, M4)+COUNTIF($F$141:$F$141, M4)+COUNTIF($F$130:$F$131, M4)+COUNTIF($F$111:$F$112, M4)+COUNTIF($F$96:$F$98, M4)&gt;1,NOT(ISBLANK(M4)))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="76" priority="1232" stopIfTrue="1">
+    <cfRule type="expression" dxfId="75" priority="1232" stopIfTrue="1">
       <formula>AND(COUNTIF($F$294:$F$65454, M4)+COUNTIF($F$1:$F$27, M4)+COUNTIF(#REF!, M4)+COUNTIF($F$252:$F$255, M4)+COUNTIF($F$229:$F$230, M4)+COUNTIF($F$202:$F$203, M4)+COUNTIF($F$181:$F$181, M4)+COUNTIF($F$166:$F$167, M4)+COUNTIF($F$141:$F$141, M4)+COUNTIF($F$130:$F$131, M4)+COUNTIF($F$111:$F$112, M4)+COUNTIF($F$96:$F$98, M4)&gt;1,NOT(ISBLANK(M4)))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="75" priority="1233" stopIfTrue="1">
+    <cfRule type="expression" dxfId="74" priority="1233" stopIfTrue="1">
       <formula>AND(COUNTIF($F$252:$F$65454, M4)+COUNTIF(#REF!, M4)+COUNTIF($F$1:$F$27, M4)+COUNTIF($F$229:$F$230, M4)+COUNTIF($F$202:$F$203, M4)+COUNTIF($F$181:$F$181, M4)+COUNTIF($F$166:$F$167, M4)+COUNTIF($F$141:$F$141, M4)+COUNTIF($F$130:$F$131, M4)+COUNTIF($F$111:$F$112, M4)+COUNTIF($F$96:$F$98, M4)&gt;1,NOT(ISBLANK(M4)))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="74" priority="1234" stopIfTrue="1">
+    <cfRule type="expression" dxfId="73" priority="1234" stopIfTrue="1">
       <formula>AND(COUNTIF($F$252:$F$65454, M4)+COUNTIF($F$229:$F$230, M4)+COUNTIF($F$202:$F$203, M4)+COUNTIF($F$181:$F$181, M4)+COUNTIF($F$166:$F$167, M4)+COUNTIF($F$1:$F$27, M4)+COUNTIF(#REF!, M4)+COUNTIF($F$141:$F$141, M4)+COUNTIF($F$130:$F$131, M4)+COUNTIF(#REF!, M4)+COUNTIF($F$111:$F$112, M4)+COUNTIF($F$89:$F$89, M4)+COUNTIF($F$91:$F$98, M4)+COUNTIF(#REF!, M4)&gt;1,NOT(ISBLANK(M4)))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="73" priority="1235" stopIfTrue="1">
+    <cfRule type="expression" dxfId="72" priority="1235" stopIfTrue="1">
       <formula>AND(COUNTIF($F$229:$F$65454, M4)+COUNTIF($F$202:$F$203, M4)+COUNTIF($F$181:$F$181, M4)+COUNTIF($F$166:$F$167, M4)+COUNTIF($F$1:$F$27, M4)+COUNTIF(#REF!, M4)+COUNTIF($F$141:$F$141, M4)+COUNTIF($F$130:$F$131, M4)+COUNTIF(#REF!, M4)+COUNTIF($F$111:$F$112, M4)+COUNTIF($F$89:$F$89, M4)+COUNTIF($F$91:$F$98, M4)+COUNTIF(#REF!, M4)&gt;1,NOT(ISBLANK(M4)))</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="72" priority="1222" stopIfTrue="1">
-      <formula>AND(COUNTIF($D$331:$D$65460, M4)+COUNTIF($D$1:$D$27, M4)+COUNTIF(#REF!, M4)+COUNTIF($D$314:$D$315, M4)+COUNTIF($D$294:$D$295, M4)+COUNTIF($D$256:$D$257, M4)+COUNTIF($D$214:$D$217, M4)+COUNTIF($D$191:$D$192, M4)+COUNTIF($D$164:$D$165, M4)+COUNTIF($D$143:$D$143, M4)+COUNTIF($D$128:$D$129, M4)+COUNTIF($D$103:$D$103, M4)+COUNTIF($D$92:$D$93, M4)+COUNTIF($D$73:$D$74, M4)+COUNTIF($D$58:$D$60, M4)&gt;1,NOT(ISBLANK(M4)))</formula>
     </cfRule>
   </conditionalFormatting>
   <printOptions horizontalCentered="1"/>
@@ -4895,7 +4895,7 @@
       <c r="Q4" s="70">
         <v>0</v>
       </c>
-      <c r="R4" s="182" t="s">
+      <c r="R4" s="198" t="s">
         <v>75</v>
       </c>
     </row>
@@ -4938,14 +4938,14 @@
       <c r="Q5" s="70">
         <v>0</v>
       </c>
-      <c r="R5" s="183"/>
+      <c r="R5" s="199"/>
     </row>
     <row r="6" spans="2:18" s="75" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="B6" s="184" t="s">
+      <c r="B6" s="200" t="s">
         <v>29</v>
       </c>
-      <c r="C6" s="185"/>
-      <c r="D6" s="186"/>
+      <c r="C6" s="201"/>
+      <c r="D6" s="202"/>
       <c r="E6" s="73">
         <v>160</v>
       </c>
@@ -7005,28 +7005,28 @@
     <cfRule type="duplicateValues" dxfId="61" priority="160"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="J2:J14 K16 J16:J31">
-    <cfRule type="containsText" dxfId="60" priority="197" operator="containsText" text="Complete">
+    <cfRule type="containsText" dxfId="60" priority="179" operator="containsText" text="WIP">
+      <formula>NOT(ISERROR(SEARCH("WIP",J2)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="59" priority="182" operator="containsText" text="Complete">
       <formula>NOT(ISERROR(SEARCH("Complete",J2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="59" priority="198" operator="containsText" text="ROW">
+    <cfRule type="containsText" dxfId="58" priority="183" operator="containsText" text="ROW">
       <formula>NOT(ISERROR(SEARCH("ROW",J2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="58" priority="179" operator="containsText" text="WIP">
-      <formula>NOT(ISERROR(SEARCH("WIP",J2)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="57" priority="182" operator="containsText" text="Complete">
+    <cfRule type="containsText" dxfId="57" priority="197" operator="containsText" text="Complete">
       <formula>NOT(ISERROR(SEARCH("Complete",J2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="56" priority="183" operator="containsText" text="ROW">
+    <cfRule type="containsText" dxfId="56" priority="198" operator="containsText" text="ROW">
       <formula>NOT(ISERROR(SEARCH("ROW",J2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K3:K7 K9:K13 K20:K22">
-    <cfRule type="containsText" dxfId="55" priority="112" operator="containsText" text="ROW">
+    <cfRule type="containsText" dxfId="55" priority="111" operator="containsText" text="Complete">
+      <formula>NOT(ISERROR(SEARCH("Complete",K3)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="54" priority="112" operator="containsText" text="ROW">
       <formula>NOT(ISERROR(SEARCH("ROW",K3)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="54" priority="111" operator="containsText" text="Complete">
-      <formula>NOT(ISERROR(SEARCH("Complete",K3)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K3:K7 K9:K13 K20:N22">
@@ -7072,14 +7072,14 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L15">
-    <cfRule type="containsText" dxfId="43" priority="3" operator="containsText" text="ROW">
-      <formula>NOT(ISERROR(SEARCH("ROW",L15)))</formula>
+    <cfRule type="containsText" dxfId="43" priority="1" operator="containsText" text="WIP">
+      <formula>NOT(ISERROR(SEARCH("WIP",L15)))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="42" priority="2" operator="containsText" text="Complete">
       <formula>NOT(ISERROR(SEARCH("Complete",L15)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="41" priority="1" operator="containsText" text="WIP">
-      <formula>NOT(ISERROR(SEARCH("WIP",L15)))</formula>
+    <cfRule type="containsText" dxfId="41" priority="3" operator="containsText" text="ROW">
+      <formula>NOT(ISERROR(SEARCH("ROW",L15)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L2:N7 J2:J14 L8:M8 L9:N14 N15 K16:M16 J16:J27 K17:N18 L23:N26 O24 K25:K26 O26:O30 K27:N27 J28:N31">
@@ -7093,11 +7093,11 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L19:N19">
-    <cfRule type="containsText" dxfId="38" priority="18" operator="containsText" text="ROW">
+    <cfRule type="containsText" dxfId="38" priority="17" operator="containsText" text="Complete">
+      <formula>NOT(ISERROR(SEARCH("Complete",L19)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="37" priority="18" operator="containsText" text="ROW">
       <formula>NOT(ISERROR(SEARCH("ROW",L19)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="37" priority="17" operator="containsText" text="Complete">
-      <formula>NOT(ISERROR(SEARCH("Complete",L19)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L19:O19">
@@ -7117,11 +7117,11 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O3:O8">
-    <cfRule type="containsText" dxfId="32" priority="37" operator="containsText" text="ROW">
+    <cfRule type="containsText" dxfId="32" priority="36" operator="containsText" text="Complete">
+      <formula>NOT(ISERROR(SEARCH("Complete",O3)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="31" priority="37" operator="containsText" text="ROW">
       <formula>NOT(ISERROR(SEARCH("ROW",O3)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="31" priority="36" operator="containsText" text="Complete">
-      <formula>NOT(ISERROR(SEARCH("Complete",O3)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O4">
@@ -7146,25 +7146,25 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O9">
-    <cfRule type="containsText" dxfId="25" priority="28" operator="containsText" text="ROW">
+    <cfRule type="containsText" dxfId="25" priority="26" operator="containsText" text="WIP">
+      <formula>NOT(ISERROR(SEARCH("WIP",O9)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="24" priority="27" operator="containsText" text="Complete">
+      <formula>NOT(ISERROR(SEARCH("Complete",O9)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="23" priority="28" operator="containsText" text="ROW">
       <formula>NOT(ISERROR(SEARCH("ROW",O9)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="24" priority="26" operator="containsText" text="WIP">
-      <formula>NOT(ISERROR(SEARCH("WIP",O9)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="23" priority="27" operator="containsText" text="Complete">
-      <formula>NOT(ISERROR(SEARCH("Complete",O9)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O10">
-    <cfRule type="containsText" dxfId="22" priority="59" operator="containsText" text="ROW">
+    <cfRule type="containsText" dxfId="22" priority="57" operator="containsText" text="WIP">
+      <formula>NOT(ISERROR(SEARCH("WIP",O10)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="21" priority="58" operator="containsText" text="Complete">
+      <formula>NOT(ISERROR(SEARCH("Complete",O10)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="20" priority="59" operator="containsText" text="ROW">
       <formula>NOT(ISERROR(SEARCH("ROW",O10)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="21" priority="57" operator="containsText" text="WIP">
-      <formula>NOT(ISERROR(SEARCH("WIP",O10)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="20" priority="58" operator="containsText" text="Complete">
-      <formula>NOT(ISERROR(SEARCH("Complete",O10)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O10:O13">
@@ -7181,19 +7181,19 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O13">
-    <cfRule type="containsText" dxfId="16" priority="25" operator="containsText" text="ROW">
+    <cfRule type="containsText" dxfId="16" priority="24" operator="containsText" text="Complete">
+      <formula>NOT(ISERROR(SEARCH("Complete",O13)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="15" priority="25" operator="containsText" text="ROW">
       <formula>NOT(ISERROR(SEARCH("ROW",O13)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="15" priority="24" operator="containsText" text="Complete">
-      <formula>NOT(ISERROR(SEARCH("Complete",O13)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O13:O14">
-    <cfRule type="containsText" dxfId="14" priority="53" operator="containsText" text="ROW">
+    <cfRule type="containsText" dxfId="14" priority="52" operator="containsText" text="Complete">
+      <formula>NOT(ISERROR(SEARCH("Complete",O13)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="13" priority="53" operator="containsText" text="ROW">
       <formula>NOT(ISERROR(SEARCH("ROW",O13)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="13" priority="52" operator="containsText" text="Complete">
-      <formula>NOT(ISERROR(SEARCH("Complete",O13)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O13:O17">
@@ -7210,11 +7210,11 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O15:O17">
-    <cfRule type="containsText" dxfId="9" priority="13" operator="containsText" text="ROW">
+    <cfRule type="containsText" dxfId="9" priority="12" operator="containsText" text="Complete">
+      <formula>NOT(ISERROR(SEARCH("Complete",O15)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="8" priority="13" operator="containsText" text="ROW">
       <formula>NOT(ISERROR(SEARCH("ROW",O15)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="8" priority="12" operator="containsText" text="Complete">
-      <formula>NOT(ISERROR(SEARCH("Complete",O15)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O19:O20">
@@ -7255,89 +7255,89 @@
   <dimension ref="A1:O11"/>
   <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="13" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="12" style="191" customWidth="1"/>
-    <col min="2" max="2" width="10.81640625" style="191" customWidth="1"/>
-    <col min="3" max="3" width="28.7265625" style="191" customWidth="1"/>
-    <col min="4" max="4" width="21.7265625" style="191" customWidth="1"/>
-    <col min="5" max="5" width="24.26953125" style="191" customWidth="1"/>
-    <col min="6" max="6" width="19.453125" style="191" customWidth="1"/>
-    <col min="7" max="7" width="19.1796875" style="191" customWidth="1"/>
-    <col min="8" max="8" width="19.26953125" style="191" customWidth="1"/>
-    <col min="9" max="9" width="25.7265625" style="191" customWidth="1"/>
-    <col min="10" max="10" width="25.1796875" style="191" customWidth="1"/>
-    <col min="11" max="11" width="17.1796875" style="191" customWidth="1"/>
-    <col min="12" max="12" width="22.54296875" style="191" customWidth="1"/>
-    <col min="13" max="13" width="26.81640625" style="191" customWidth="1"/>
-    <col min="14" max="14" width="41.7265625" style="191" customWidth="1"/>
-    <col min="15" max="15" width="23.1796875" style="191" customWidth="1"/>
-    <col min="16" max="16384" width="9.1796875" style="191"/>
+    <col min="1" max="1" width="12" style="161" customWidth="1"/>
+    <col min="2" max="2" width="10.81640625" style="161" customWidth="1"/>
+    <col min="3" max="3" width="28.7265625" style="161" customWidth="1"/>
+    <col min="4" max="4" width="21.7265625" style="161" customWidth="1"/>
+    <col min="5" max="5" width="24.26953125" style="161" customWidth="1"/>
+    <col min="6" max="6" width="19.453125" style="161" customWidth="1"/>
+    <col min="7" max="7" width="19.1796875" style="161" customWidth="1"/>
+    <col min="8" max="8" width="19.26953125" style="161" customWidth="1"/>
+    <col min="9" max="9" width="25.7265625" style="161" customWidth="1"/>
+    <col min="10" max="10" width="25.1796875" style="161" customWidth="1"/>
+    <col min="11" max="11" width="17.1796875" style="161" customWidth="1"/>
+    <col min="12" max="12" width="22.54296875" style="161" customWidth="1"/>
+    <col min="13" max="13" width="26.81640625" style="161" customWidth="1"/>
+    <col min="14" max="14" width="41.7265625" style="161" customWidth="1"/>
+    <col min="15" max="15" width="23.1796875" style="161" customWidth="1"/>
+    <col min="16" max="16384" width="9.1796875" style="161"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="14.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="2" spans="1:15" ht="55.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="192" t="s">
+      <c r="A2" s="162" t="s">
         <v>180</v>
       </c>
-      <c r="B2" s="193" t="s">
+      <c r="B2" s="163" t="s">
         <v>181</v>
       </c>
-      <c r="C2" s="194" t="s">
+      <c r="C2" s="164" t="s">
         <v>182</v>
       </c>
-      <c r="D2" s="193" t="s">
+      <c r="D2" s="163" t="s">
         <v>183</v>
       </c>
-      <c r="E2" s="193" t="s">
+      <c r="E2" s="163" t="s">
         <v>184</v>
       </c>
-      <c r="F2" s="193" t="s">
+      <c r="F2" s="163" t="s">
         <v>185</v>
       </c>
-      <c r="G2" s="193" t="s">
+      <c r="G2" s="163" t="s">
         <v>186</v>
       </c>
-      <c r="H2" s="193" t="s">
+      <c r="H2" s="163" t="s">
         <v>187</v>
       </c>
-      <c r="I2" s="193" t="s">
+      <c r="I2" s="163" t="s">
         <v>188</v>
       </c>
-      <c r="J2" s="193" t="s">
+      <c r="J2" s="163" t="s">
         <v>189</v>
       </c>
-      <c r="K2" s="195" t="s">
+      <c r="K2" s="165" t="s">
         <v>190</v>
       </c>
-      <c r="L2" s="195" t="s">
+      <c r="L2" s="165" t="s">
         <v>109</v>
       </c>
-      <c r="M2" s="196" t="s">
+      <c r="M2" s="166" t="s">
         <v>191</v>
       </c>
-      <c r="N2" s="197" t="s">
+      <c r="N2" s="167" t="s">
         <v>105</v>
       </c>
-      <c r="O2" s="198" t="s">
+      <c r="O2" s="168" t="s">
         <v>104</v>
       </c>
     </row>
     <row r="3" spans="1:15" ht="66.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="199">
+      <c r="A3" s="169">
         <v>1</v>
       </c>
-      <c r="B3" s="200" t="s">
+      <c r="B3" s="170" t="s">
         <v>192</v>
       </c>
       <c r="C3" s="4" t="s">
         <v>193</v>
       </c>
       <c r="D3" s="8">
-        <v>1.5389999999999999</v>
-      </c>
-      <c r="E3" s="201" t="s">
+        <v>1539</v>
+      </c>
+      <c r="E3" s="171" t="s">
         <v>176</v>
       </c>
-      <c r="F3" s="199">
+      <c r="F3" s="169">
         <v>5</v>
       </c>
       <c r="G3" s="114">
@@ -7349,42 +7349,42 @@
       <c r="I3" s="114">
         <v>45974</v>
       </c>
-      <c r="J3" s="202">
+      <c r="J3" s="172">
         <v>45976</v>
       </c>
-      <c r="K3" s="203" t="s">
+      <c r="K3" s="173" t="s">
         <v>194</v>
       </c>
-      <c r="L3" s="204" t="s">
+      <c r="L3" s="174" t="s">
         <v>195</v>
       </c>
-      <c r="M3" s="204">
+      <c r="M3" s="174">
         <v>40</v>
       </c>
-      <c r="N3" s="199" t="s">
+      <c r="N3" s="169" t="s">
         <v>196</v>
       </c>
-      <c r="O3" s="199" t="s">
+      <c r="O3" s="169" t="s">
         <v>197</v>
       </c>
     </row>
     <row r="4" spans="1:15" ht="63" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="199">
+      <c r="A4" s="169">
         <v>2</v>
       </c>
-      <c r="B4" s="200" t="s">
+      <c r="B4" s="170" t="s">
         <v>198</v>
       </c>
       <c r="C4" s="8" t="s">
         <v>192</v>
       </c>
       <c r="D4" s="8">
-        <v>4.7619999999999996</v>
-      </c>
-      <c r="E4" s="201" t="s">
+        <v>4762</v>
+      </c>
+      <c r="E4" s="171" t="s">
         <v>199</v>
       </c>
-      <c r="F4" s="199">
+      <c r="F4" s="169">
         <v>12</v>
       </c>
       <c r="G4" s="156">
@@ -7396,42 +7396,42 @@
       <c r="I4" s="114">
         <v>45981</v>
       </c>
-      <c r="J4" s="202">
+      <c r="J4" s="172">
         <v>45984</v>
       </c>
-      <c r="K4" s="203" t="s">
+      <c r="K4" s="173" t="s">
         <v>194</v>
       </c>
-      <c r="L4" s="204" t="s">
+      <c r="L4" s="174" t="s">
         <v>195</v>
       </c>
-      <c r="M4" s="204">
+      <c r="M4" s="174">
         <v>40</v>
       </c>
-      <c r="N4" s="199" t="s">
+      <c r="N4" s="169" t="s">
         <v>196</v>
       </c>
-      <c r="O4" s="199" t="s">
+      <c r="O4" s="169" t="s">
         <v>197</v>
       </c>
     </row>
     <row r="5" spans="1:15" ht="63" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="199">
+      <c r="A5" s="169">
         <v>3</v>
       </c>
-      <c r="B5" s="200" t="s">
+      <c r="B5" s="170" t="s">
         <v>200</v>
       </c>
       <c r="C5" s="8" t="s">
         <v>198</v>
       </c>
       <c r="D5" s="8">
-        <v>1.909</v>
-      </c>
-      <c r="E5" s="201" t="s">
+        <v>1909</v>
+      </c>
+      <c r="E5" s="171" t="s">
         <v>176</v>
       </c>
-      <c r="F5" s="199">
+      <c r="F5" s="169">
         <v>5</v>
       </c>
       <c r="G5" s="114">
@@ -7443,42 +7443,42 @@
       <c r="I5" s="114">
         <v>45985</v>
       </c>
-      <c r="J5" s="202">
+      <c r="J5" s="172">
         <v>45988</v>
       </c>
-      <c r="K5" s="203" t="s">
+      <c r="K5" s="173" t="s">
         <v>194</v>
       </c>
-      <c r="L5" s="204" t="s">
+      <c r="L5" s="174" t="s">
         <v>195</v>
       </c>
-      <c r="M5" s="204">
+      <c r="M5" s="174">
         <v>40</v>
       </c>
-      <c r="N5" s="199" t="s">
+      <c r="N5" s="169" t="s">
         <v>196</v>
       </c>
-      <c r="O5" s="199" t="s">
+      <c r="O5" s="169" t="s">
         <v>197</v>
       </c>
     </row>
     <row r="6" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="199">
+      <c r="A6" s="169">
         <v>4</v>
       </c>
-      <c r="B6" s="200" t="s">
+      <c r="B6" s="170" t="s">
         <v>201</v>
       </c>
       <c r="C6" s="8" t="s">
         <v>202</v>
       </c>
       <c r="D6" s="8">
-        <v>0.248</v>
-      </c>
-      <c r="E6" s="201" t="s">
+        <v>248</v>
+      </c>
+      <c r="E6" s="171" t="s">
         <v>176</v>
       </c>
-      <c r="F6" s="199">
+      <c r="F6" s="169">
         <v>2</v>
       </c>
       <c r="G6" s="114">
@@ -7490,42 +7490,42 @@
       <c r="I6" s="114">
         <v>45991</v>
       </c>
-      <c r="J6" s="202">
+      <c r="J6" s="172">
         <v>45991</v>
       </c>
-      <c r="K6" s="205" t="s">
+      <c r="K6" s="175" t="s">
         <v>203</v>
       </c>
-      <c r="L6" s="204" t="s">
+      <c r="L6" s="174" t="s">
         <v>195</v>
       </c>
-      <c r="M6" s="204">
+      <c r="M6" s="174">
         <v>40</v>
       </c>
-      <c r="N6" s="199" t="s">
+      <c r="N6" s="169" t="s">
         <v>196</v>
       </c>
-      <c r="O6" s="199" t="s">
+      <c r="O6" s="169" t="s">
         <v>197</v>
       </c>
     </row>
     <row r="7" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="199">
+      <c r="A7" s="169">
         <v>5</v>
       </c>
-      <c r="B7" s="200" t="s">
+      <c r="B7" s="170" t="s">
         <v>202</v>
       </c>
       <c r="C7" s="8" t="s">
         <v>204</v>
       </c>
       <c r="D7" s="8">
-        <v>0.43</v>
-      </c>
-      <c r="E7" s="201" t="s">
+        <v>430</v>
+      </c>
+      <c r="E7" s="171" t="s">
         <v>176</v>
       </c>
-      <c r="F7" s="199">
+      <c r="F7" s="169">
         <v>1</v>
       </c>
       <c r="G7" s="114">
@@ -7537,42 +7537,42 @@
       <c r="I7" s="114">
         <v>45991</v>
       </c>
-      <c r="J7" s="202">
+      <c r="J7" s="172">
         <v>45991</v>
       </c>
-      <c r="K7" s="205" t="s">
+      <c r="K7" s="175" t="s">
         <v>203</v>
       </c>
-      <c r="L7" s="204" t="s">
+      <c r="L7" s="174" t="s">
         <v>195</v>
       </c>
-      <c r="M7" s="204">
+      <c r="M7" s="174">
         <v>40</v>
       </c>
-      <c r="N7" s="199" t="s">
+      <c r="N7" s="169" t="s">
         <v>196</v>
       </c>
-      <c r="O7" s="199" t="s">
+      <c r="O7" s="169" t="s">
         <v>197</v>
       </c>
     </row>
     <row r="8" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="199">
+      <c r="A8" s="169">
         <v>6</v>
       </c>
-      <c r="B8" s="200" t="s">
+      <c r="B8" s="170" t="s">
         <v>204</v>
       </c>
       <c r="C8" s="8" t="s">
         <v>205</v>
       </c>
       <c r="D8" s="8">
-        <v>0.248</v>
-      </c>
-      <c r="E8" s="201" t="s">
+        <v>248</v>
+      </c>
+      <c r="E8" s="171" t="s">
         <v>176</v>
       </c>
-      <c r="F8" s="199">
+      <c r="F8" s="169">
         <v>1</v>
       </c>
       <c r="G8" s="114">
@@ -7584,42 +7584,42 @@
       <c r="I8" s="114">
         <v>45991</v>
       </c>
-      <c r="J8" s="202">
+      <c r="J8" s="172">
         <v>45991</v>
       </c>
-      <c r="K8" s="205" t="s">
+      <c r="K8" s="175" t="s">
         <v>203</v>
       </c>
-      <c r="L8" s="204" t="s">
+      <c r="L8" s="174" t="s">
         <v>195</v>
       </c>
-      <c r="M8" s="204">
+      <c r="M8" s="174">
         <v>40</v>
       </c>
-      <c r="N8" s="199" t="s">
+      <c r="N8" s="169" t="s">
         <v>196</v>
       </c>
-      <c r="O8" s="199" t="s">
+      <c r="O8" s="169" t="s">
         <v>197</v>
       </c>
     </row>
     <row r="9" spans="1:15" ht="68.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="199">
+      <c r="A9" s="169">
         <v>7</v>
       </c>
-      <c r="B9" s="200" t="s">
+      <c r="B9" s="170" t="s">
         <v>206</v>
       </c>
       <c r="C9" s="8" t="s">
         <v>207</v>
       </c>
       <c r="D9" s="8">
-        <v>4.91</v>
-      </c>
-      <c r="E9" s="201" t="s">
+        <v>4910</v>
+      </c>
+      <c r="E9" s="171" t="s">
         <v>176</v>
       </c>
-      <c r="F9" s="199">
+      <c r="F9" s="169">
         <v>12</v>
       </c>
       <c r="G9" s="114">
@@ -7631,42 +7631,42 @@
       <c r="I9" s="114">
         <v>45976</v>
       </c>
-      <c r="J9" s="202">
+      <c r="J9" s="172">
         <v>45979</v>
       </c>
-      <c r="K9" s="205" t="s">
+      <c r="K9" s="175" t="s">
         <v>208</v>
       </c>
-      <c r="L9" s="199" t="s">
+      <c r="L9" s="169" t="s">
         <v>209</v>
       </c>
-      <c r="M9" s="199">
+      <c r="M9" s="169">
         <v>45</v>
       </c>
-      <c r="N9" s="199" t="s">
+      <c r="N9" s="169" t="s">
         <v>210</v>
       </c>
-      <c r="O9" s="199" t="s">
+      <c r="O9" s="169" t="s">
         <v>211</v>
       </c>
     </row>
     <row r="10" spans="1:15" ht="76.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="199">
+      <c r="A10" s="169">
         <v>8</v>
       </c>
-      <c r="B10" s="200" t="s">
+      <c r="B10" s="170" t="s">
         <v>207</v>
       </c>
       <c r="C10" s="8" t="s">
         <v>200</v>
       </c>
       <c r="D10" s="8">
-        <v>0.498</v>
-      </c>
-      <c r="E10" s="201" t="s">
+        <v>498</v>
+      </c>
+      <c r="E10" s="171" t="s">
         <v>176</v>
       </c>
-      <c r="F10" s="199">
+      <c r="F10" s="169">
         <v>1</v>
       </c>
       <c r="G10" s="114">
@@ -7678,42 +7678,42 @@
       <c r="I10" s="114">
         <v>45978</v>
       </c>
-      <c r="J10" s="202">
+      <c r="J10" s="172">
         <v>45981</v>
       </c>
-      <c r="K10" s="205" t="s">
+      <c r="K10" s="175" t="s">
         <v>208</v>
       </c>
-      <c r="L10" s="199" t="s">
+      <c r="L10" s="169" t="s">
         <v>209</v>
       </c>
-      <c r="M10" s="199">
+      <c r="M10" s="169">
         <v>45</v>
       </c>
-      <c r="N10" s="199" t="s">
+      <c r="N10" s="169" t="s">
         <v>210</v>
       </c>
-      <c r="O10" s="199" t="s">
+      <c r="O10" s="169" t="s">
         <v>211</v>
       </c>
     </row>
     <row r="11" spans="1:15" ht="63" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="199">
+      <c r="A11" s="169">
         <v>9</v>
       </c>
-      <c r="B11" s="200" t="s">
+      <c r="B11" s="170" t="s">
         <v>212</v>
       </c>
       <c r="C11" s="8" t="s">
         <v>213</v>
       </c>
       <c r="D11" s="8">
-        <v>4.7510000000000003</v>
-      </c>
-      <c r="E11" s="206" t="s">
+        <v>4751</v>
+      </c>
+      <c r="E11" s="176" t="s">
         <v>214</v>
       </c>
-      <c r="F11" s="199">
+      <c r="F11" s="169">
         <v>11</v>
       </c>
       <c r="G11" s="114">
@@ -7725,22 +7725,22 @@
       <c r="I11" s="114">
         <v>45991</v>
       </c>
-      <c r="J11" s="202">
+      <c r="J11" s="172">
         <v>45991</v>
       </c>
-      <c r="K11" s="205" t="s">
+      <c r="K11" s="175" t="s">
         <v>208</v>
       </c>
-      <c r="L11" s="199" t="s">
+      <c r="L11" s="169" t="s">
         <v>209</v>
       </c>
-      <c r="M11" s="199">
+      <c r="M11" s="169">
         <v>45</v>
       </c>
-      <c r="N11" s="199" t="s">
+      <c r="N11" s="169" t="s">
         <v>210</v>
       </c>
-      <c r="O11" s="199" t="s">
+      <c r="O11" s="169" t="s">
         <v>211</v>
       </c>
     </row>
@@ -8018,118 +8018,118 @@
       <c r="F17" s="6"/>
     </row>
     <row r="18" spans="1:28" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="179" t="s">
+      <c r="A18" s="180" t="s">
         <v>4</v>
       </c>
-      <c r="B18" s="179" t="s">
+      <c r="B18" s="180" t="s">
         <v>42</v>
       </c>
-      <c r="C18" s="175" t="s">
+      <c r="C18" s="177" t="s">
         <v>47</v>
       </c>
-      <c r="D18" s="175" t="s">
+      <c r="D18" s="177" t="s">
         <v>43</v>
       </c>
-      <c r="E18" s="179" t="s">
+      <c r="E18" s="180" t="s">
         <v>8</v>
       </c>
-      <c r="F18" s="166" t="s">
+      <c r="F18" s="192" t="s">
         <v>18</v>
       </c>
-      <c r="G18" s="166"/>
-      <c r="H18" s="166"/>
-      <c r="I18" s="166"/>
-      <c r="J18" s="166"/>
-      <c r="K18" s="169" t="s">
+      <c r="G18" s="192"/>
+      <c r="H18" s="192"/>
+      <c r="I18" s="192"/>
+      <c r="J18" s="192"/>
+      <c r="K18" s="185" t="s">
         <v>19</v>
       </c>
-      <c r="M18" s="175" t="s">
+      <c r="M18" s="177" t="s">
         <v>36</v>
       </c>
-      <c r="O18" s="170" t="s">
+      <c r="O18" s="186" t="s">
         <v>31</v>
       </c>
-      <c r="P18" s="171"/>
-      <c r="Q18" s="171"/>
-      <c r="R18" s="171"/>
-      <c r="S18" s="171"/>
-      <c r="T18" s="172"/>
-      <c r="V18" s="170" t="s">
+      <c r="P18" s="187"/>
+      <c r="Q18" s="187"/>
+      <c r="R18" s="187"/>
+      <c r="S18" s="187"/>
+      <c r="T18" s="188"/>
+      <c r="V18" s="186" t="s">
         <v>30</v>
       </c>
-      <c r="W18" s="171"/>
-      <c r="X18" s="171"/>
-      <c r="Y18" s="171"/>
-      <c r="Z18" s="171"/>
-      <c r="AA18" s="172"/>
-      <c r="AB18" s="173" t="s">
+      <c r="W18" s="187"/>
+      <c r="X18" s="187"/>
+      <c r="Y18" s="187"/>
+      <c r="Z18" s="187"/>
+      <c r="AA18" s="188"/>
+      <c r="AB18" s="189" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="19" spans="1:28" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="180"/>
-      <c r="B19" s="180"/>
-      <c r="C19" s="177"/>
-      <c r="D19" s="180"/>
-      <c r="E19" s="180"/>
-      <c r="F19" s="187" t="s">
+      <c r="A19" s="181"/>
+      <c r="B19" s="181"/>
+      <c r="C19" s="178"/>
+      <c r="D19" s="181"/>
+      <c r="E19" s="181"/>
+      <c r="F19" s="204" t="s">
         <v>40</v>
       </c>
-      <c r="G19" s="188" t="s">
+      <c r="G19" s="205" t="s">
         <v>44</v>
       </c>
-      <c r="H19" s="189"/>
-      <c r="I19" s="188" t="s">
+      <c r="H19" s="206"/>
+      <c r="I19" s="205" t="s">
         <v>45</v>
       </c>
-      <c r="J19" s="189"/>
-      <c r="K19" s="169"/>
-      <c r="M19" s="176"/>
-      <c r="O19" s="167" t="s">
+      <c r="J19" s="206"/>
+      <c r="K19" s="185"/>
+      <c r="M19" s="191"/>
+      <c r="O19" s="183" t="s">
         <v>24</v>
       </c>
-      <c r="P19" s="167" t="s">
+      <c r="P19" s="183" t="s">
         <v>25</v>
       </c>
-      <c r="Q19" s="167" t="s">
+      <c r="Q19" s="183" t="s">
         <v>26</v>
       </c>
-      <c r="R19" s="167" t="s">
+      <c r="R19" s="183" t="s">
         <v>27</v>
       </c>
-      <c r="S19" s="167" t="s">
+      <c r="S19" s="183" t="s">
         <v>28</v>
       </c>
       <c r="T19" s="43" t="s">
         <v>29</v>
       </c>
-      <c r="V19" s="167" t="s">
+      <c r="V19" s="183" t="s">
         <v>24</v>
       </c>
-      <c r="W19" s="167" t="s">
+      <c r="W19" s="183" t="s">
         <v>25</v>
       </c>
-      <c r="X19" s="167" t="s">
+      <c r="X19" s="183" t="s">
         <v>26</v>
       </c>
-      <c r="Y19" s="167" t="s">
+      <c r="Y19" s="183" t="s">
         <v>27</v>
       </c>
-      <c r="Z19" s="167" t="s">
+      <c r="Z19" s="183" t="s">
         <v>28</v>
       </c>
       <c r="AA19" s="43" t="s">
         <v>29</v>
       </c>
-      <c r="AB19" s="174"/>
+      <c r="AB19" s="190"/>
     </row>
     <row r="20" spans="1:28" ht="36.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A20" s="180"/>
-      <c r="B20" s="180"/>
-      <c r="C20" s="177"/>
-      <c r="D20" s="180"/>
-      <c r="E20" s="180"/>
-      <c r="F20" s="187"/>
+      <c r="A20" s="181"/>
+      <c r="B20" s="181"/>
+      <c r="C20" s="178"/>
+      <c r="D20" s="181"/>
+      <c r="E20" s="181"/>
+      <c r="F20" s="204"/>
       <c r="G20" s="94" t="s">
         <v>10</v>
       </c>
@@ -8148,17 +8148,17 @@
       <c r="M20" s="18" t="s">
         <v>37</v>
       </c>
-      <c r="O20" s="168"/>
-      <c r="P20" s="168"/>
-      <c r="Q20" s="168"/>
-      <c r="R20" s="168"/>
-      <c r="S20" s="168"/>
+      <c r="O20" s="184"/>
+      <c r="P20" s="184"/>
+      <c r="Q20" s="184"/>
+      <c r="R20" s="184"/>
+      <c r="S20" s="184"/>
       <c r="T20" s="19"/>
-      <c r="V20" s="168"/>
-      <c r="W20" s="168"/>
-      <c r="X20" s="168"/>
-      <c r="Y20" s="168"/>
-      <c r="Z20" s="168"/>
+      <c r="V20" s="184"/>
+      <c r="W20" s="184"/>
+      <c r="X20" s="184"/>
+      <c r="Y20" s="184"/>
+      <c r="Z20" s="184"/>
       <c r="AA20" s="19" t="s">
         <v>20</v>
       </c>
@@ -8179,7 +8179,7 @@
       <c r="D21" s="8" t="s">
         <v>79</v>
       </c>
-      <c r="E21" s="190" t="s">
+      <c r="E21" s="203" t="s">
         <v>98</v>
       </c>
       <c r="F21" s="114">
@@ -8253,7 +8253,7 @@
       <c r="D22" s="8" t="s">
         <v>79</v>
       </c>
-      <c r="E22" s="190"/>
+      <c r="E22" s="203"/>
       <c r="F22" s="114">
         <v>45913</v>
       </c>
@@ -8325,7 +8325,7 @@
       <c r="D23" s="8" t="s">
         <v>86</v>
       </c>
-      <c r="E23" s="190"/>
+      <c r="E23" s="203"/>
       <c r="F23" s="114">
         <v>45910</v>
       </c>
@@ -8397,7 +8397,7 @@
       <c r="D24" s="8" t="s">
         <v>86</v>
       </c>
-      <c r="E24" s="190"/>
+      <c r="E24" s="203"/>
       <c r="F24" s="114">
         <v>45927</v>
       </c>
@@ -8469,7 +8469,7 @@
       <c r="D25" s="8" t="s">
         <v>86</v>
       </c>
-      <c r="E25" s="190"/>
+      <c r="E25" s="203"/>
       <c r="F25" s="114">
         <v>45915</v>
       </c>
@@ -9164,18 +9164,6 @@
     </row>
   </sheetData>
   <mergeCells count="25">
-    <mergeCell ref="E21:E25"/>
-    <mergeCell ref="W19:W20"/>
-    <mergeCell ref="K18:K19"/>
-    <mergeCell ref="M18:M19"/>
-    <mergeCell ref="O18:T18"/>
-    <mergeCell ref="V18:AA18"/>
-    <mergeCell ref="V19:V20"/>
-    <mergeCell ref="A18:A20"/>
-    <mergeCell ref="B18:B20"/>
-    <mergeCell ref="C18:C20"/>
-    <mergeCell ref="D18:D20"/>
-    <mergeCell ref="E18:E20"/>
     <mergeCell ref="AB18:AB19"/>
     <mergeCell ref="F19:F20"/>
     <mergeCell ref="G19:H19"/>
@@ -9189,6 +9177,18 @@
     <mergeCell ref="Q19:Q20"/>
     <mergeCell ref="R19:R20"/>
     <mergeCell ref="S19:S20"/>
+    <mergeCell ref="A18:A20"/>
+    <mergeCell ref="B18:B20"/>
+    <mergeCell ref="C18:C20"/>
+    <mergeCell ref="D18:D20"/>
+    <mergeCell ref="E18:E20"/>
+    <mergeCell ref="E21:E25"/>
+    <mergeCell ref="W19:W20"/>
+    <mergeCell ref="K18:K19"/>
+    <mergeCell ref="M18:M19"/>
+    <mergeCell ref="O18:T18"/>
+    <mergeCell ref="V18:AA18"/>
+    <mergeCell ref="V19:V20"/>
   </mergeCells>
   <conditionalFormatting sqref="C26:C27">
     <cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="4DT6">

</xml_diff>

<commit_message>
Remove outdated binary files and enhance project code extraction in callbacks
- Gangs and Lost Units Values showing
- Stringing plan almost done
</commit_message>
<xml_diff>
--- a/Raw Data/Micro Plans/November 2025/Micro Plan - TA-421 Nov'25.xlsx
+++ b/Raw Data/Micro Plans/November 2025/Micro Plan - TA-421 Nov'25.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kaushikb\Documents\Work\Git\Office-work-\Raw Data\Micro Plans\November 2025\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C965881B-D56B-4EDF-9D96-6A23D224259C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCEE4415-2D78-481B-8A00-29F4AB8B23A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="757" firstSheet="2" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="757" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="FDN-June25" sheetId="1" state="hidden" r:id="rId1"/>
@@ -1823,9 +1823,54 @@
     <xf numFmtId="0" fontId="25" fillId="0" borderId="20" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" indent="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1841,51 +1886,6 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1901,9 +1901,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1911,6 +1908,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1972,6 +1972,16 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
@@ -1992,6 +2002,66 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF9C5700"/>
       </font>
       <fill>
@@ -2002,6 +2072,16 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
@@ -2032,6 +2112,16 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF006100"/>
       </font>
       <fill>
@@ -2052,6 +2142,26 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF006100"/>
       </font>
       <fill>
@@ -2072,6 +2182,16 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
@@ -2082,6 +2202,16 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF006100"/>
       </font>
       <fill>
@@ -2092,6 +2222,16 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
@@ -2112,6 +2252,46 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF9C5700"/>
       </font>
       <fill>
@@ -2122,6 +2302,26 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
@@ -2152,6 +2352,16 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF006100"/>
       </font>
       <fill>
@@ -2172,6 +2382,16 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
@@ -2192,6 +2412,16 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF9C5700"/>
       </font>
       <fill>
@@ -2202,6 +2432,16 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
@@ -2222,6 +2462,16 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF9C5700"/>
       </font>
       <fill>
@@ -2232,6 +2482,16 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
@@ -2242,6 +2502,16 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF006100"/>
       </font>
       <fill>
@@ -2277,276 +2547,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2892,6 +2892,16 @@
     </dxf>
     <dxf>
       <font>
+        <color indexed="17"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor indexed="42"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color indexed="20"/>
       </font>
       <fill>
@@ -2914,16 +2924,6 @@
       <font>
         <color indexed="20"/>
       </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color indexed="17"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor indexed="42"/>
-        </patternFill>
-      </fill>
     </dxf>
     <dxf>
       <font>
@@ -3745,41 +3745,41 @@
       <c r="F17" s="6"/>
     </row>
     <row r="18" spans="1:33" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="180" t="s">
+      <c r="A18" s="195" t="s">
         <v>4</v>
       </c>
-      <c r="B18" s="180" t="s">
+      <c r="B18" s="195" t="s">
         <v>5</v>
       </c>
-      <c r="C18" s="177" t="s">
+      <c r="C18" s="191" t="s">
         <v>6</v>
       </c>
-      <c r="D18" s="180" t="s">
+      <c r="D18" s="195" t="s">
         <v>7</v>
       </c>
-      <c r="E18" s="177" t="s">
+      <c r="E18" s="191" t="s">
         <v>16</v>
       </c>
-      <c r="F18" s="177" t="s">
+      <c r="F18" s="191" t="s">
         <v>17</v>
       </c>
-      <c r="G18" s="180" t="s">
+      <c r="G18" s="195" t="s">
         <v>8</v>
       </c>
-      <c r="H18" s="192" t="s">
+      <c r="H18" s="182" t="s">
         <v>18</v>
       </c>
-      <c r="I18" s="192"/>
-      <c r="J18" s="192"/>
-      <c r="K18" s="192"/>
-      <c r="L18" s="192"/>
-      <c r="M18" s="192"/>
-      <c r="N18" s="192"/>
-      <c r="O18" s="192"/>
+      <c r="I18" s="182"/>
+      <c r="J18" s="182"/>
+      <c r="K18" s="182"/>
+      <c r="L18" s="182"/>
+      <c r="M18" s="182"/>
+      <c r="N18" s="182"/>
+      <c r="O18" s="182"/>
       <c r="P18" s="185" t="s">
         <v>19</v>
       </c>
-      <c r="R18" s="177" t="s">
+      <c r="R18" s="191" t="s">
         <v>36</v>
       </c>
       <c r="T18" s="186" t="s">
@@ -3803,33 +3803,33 @@
       </c>
     </row>
     <row r="19" spans="1:33" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="181"/>
-      <c r="B19" s="181"/>
-      <c r="C19" s="178"/>
-      <c r="D19" s="181"/>
-      <c r="E19" s="178"/>
-      <c r="F19" s="178"/>
-      <c r="G19" s="181"/>
-      <c r="H19" s="197" t="s">
+      <c r="A19" s="196"/>
+      <c r="B19" s="196"/>
+      <c r="C19" s="193"/>
+      <c r="D19" s="196"/>
+      <c r="E19" s="193"/>
+      <c r="F19" s="193"/>
+      <c r="G19" s="196"/>
+      <c r="H19" s="181" t="s">
         <v>9</v>
       </c>
-      <c r="I19" s="197"/>
-      <c r="J19" s="197" t="s">
+      <c r="I19" s="181"/>
+      <c r="J19" s="181" t="s">
         <v>12</v>
       </c>
-      <c r="K19" s="197"/>
-      <c r="L19" s="197" t="s">
+      <c r="K19" s="181"/>
+      <c r="L19" s="181" t="s">
         <v>13</v>
       </c>
-      <c r="M19" s="197"/>
-      <c r="N19" s="193" t="s">
+      <c r="M19" s="181"/>
+      <c r="N19" s="179" t="s">
         <v>15</v>
       </c>
-      <c r="O19" s="193" t="s">
+      <c r="O19" s="179" t="s">
         <v>14</v>
       </c>
       <c r="P19" s="185"/>
-      <c r="R19" s="191"/>
+      <c r="R19" s="192"/>
       <c r="T19" s="183" t="s">
         <v>24</v>
       </c>
@@ -3869,13 +3869,13 @@
       <c r="AG19" s="190"/>
     </row>
     <row r="20" spans="1:33" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A20" s="182"/>
-      <c r="B20" s="181"/>
-      <c r="C20" s="178"/>
-      <c r="D20" s="181"/>
-      <c r="E20" s="179"/>
-      <c r="F20" s="179"/>
-      <c r="G20" s="181"/>
+      <c r="A20" s="197"/>
+      <c r="B20" s="196"/>
+      <c r="C20" s="193"/>
+      <c r="D20" s="196"/>
+      <c r="E20" s="194"/>
+      <c r="F20" s="194"/>
+      <c r="G20" s="196"/>
       <c r="H20" s="94" t="s">
         <v>10</v>
       </c>
@@ -3894,8 +3894,8 @@
       <c r="M20" s="94" t="s">
         <v>11</v>
       </c>
-      <c r="N20" s="194"/>
-      <c r="O20" s="194"/>
+      <c r="N20" s="180"/>
+      <c r="O20" s="180"/>
       <c r="P20" s="44" t="s">
         <v>50</v>
       </c>
@@ -4183,7 +4183,7 @@
       <c r="D25" s="86"/>
       <c r="E25" s="101"/>
       <c r="F25" s="8"/>
-      <c r="G25" s="195"/>
+      <c r="G25" s="177"/>
       <c r="H25" s="99"/>
       <c r="I25" s="99"/>
       <c r="J25" s="99"/>
@@ -4241,7 +4241,7 @@
       <c r="D26" s="8"/>
       <c r="E26" s="102"/>
       <c r="F26" s="97"/>
-      <c r="G26" s="196"/>
+      <c r="G26" s="178"/>
       <c r="H26" s="99"/>
       <c r="I26" s="99"/>
       <c r="J26" s="99"/>
@@ -4596,16 +4596,13 @@
     <filterColumn colId="13" showButton="0"/>
   </autoFilter>
   <mergeCells count="29">
-    <mergeCell ref="G25:G26"/>
-    <mergeCell ref="O19:O20"/>
-    <mergeCell ref="H19:I19"/>
-    <mergeCell ref="J19:K19"/>
-    <mergeCell ref="L19:M19"/>
-    <mergeCell ref="H18:O18"/>
-    <mergeCell ref="N19:N20"/>
-    <mergeCell ref="U19:U20"/>
-    <mergeCell ref="V19:V20"/>
-    <mergeCell ref="W19:W20"/>
+    <mergeCell ref="F18:F20"/>
+    <mergeCell ref="G18:G20"/>
+    <mergeCell ref="A18:A20"/>
+    <mergeCell ref="B18:B20"/>
+    <mergeCell ref="C18:C20"/>
+    <mergeCell ref="D18:D20"/>
+    <mergeCell ref="E18:E20"/>
     <mergeCell ref="X19:X20"/>
     <mergeCell ref="P18:P19"/>
     <mergeCell ref="AA18:AF18"/>
@@ -4618,13 +4615,16 @@
     <mergeCell ref="R18:R19"/>
     <mergeCell ref="T18:Y18"/>
     <mergeCell ref="T19:T20"/>
-    <mergeCell ref="F18:F20"/>
-    <mergeCell ref="G18:G20"/>
-    <mergeCell ref="A18:A20"/>
-    <mergeCell ref="B18:B20"/>
-    <mergeCell ref="C18:C20"/>
-    <mergeCell ref="D18:D20"/>
-    <mergeCell ref="E18:E20"/>
+    <mergeCell ref="H18:O18"/>
+    <mergeCell ref="N19:N20"/>
+    <mergeCell ref="U19:U20"/>
+    <mergeCell ref="V19:V20"/>
+    <mergeCell ref="W19:W20"/>
+    <mergeCell ref="G25:G26"/>
+    <mergeCell ref="O19:O20"/>
+    <mergeCell ref="H19:I19"/>
+    <mergeCell ref="J19:K19"/>
+    <mergeCell ref="L19:M19"/>
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B21">
@@ -4699,17 +4699,17 @@
     <cfRule type="expression" dxfId="99" priority="1243" stopIfTrue="1">
       <formula>AND(COUNTIF($D$1:$D$123, B26)+COUNTIF($D$142:$D$65380, B26)&gt;1,NOT(ISBLANK(B26)))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="98" priority="1244" stopIfTrue="1">
+    <cfRule type="expression" dxfId="98" priority="1245" stopIfTrue="1">
       <formula>AND(COUNTIF($D$1:$D$191, B26)+COUNTIF($D$214:$D$65380, B26)&gt;1,NOT(ISBLANK(B26)))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="97" priority="1245" stopIfTrue="1">
+    <cfRule type="expression" dxfId="97" priority="1246" stopIfTrue="1">
       <formula>AND(COUNTIF($D$1:$D$191, B26)+COUNTIF($D$214:$D$65380, B26)&gt;1,NOT(ISBLANK(B26)))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="96" priority="1246" stopIfTrue="1">
+    <cfRule type="expression" dxfId="96" priority="1247" stopIfTrue="1">
+      <formula>AND(COUNTIF($D$474:$D$65380, B26)+COUNTIF($D$454:$D$455, B26)+COUNTIF($D$416:$D$417, B26)+COUNTIF($D$374:$D$377, B26)+COUNTIF($D$351:$D$352, B26)+COUNTIF($D$324:$D$325, B26)+COUNTIF($D$303:$D$303, B26)+COUNTIF($D$288:$D$289, B26)+COUNTIF($D$263:$D$263, B26)+COUNTIF($D$252:$D$253, B26)+COUNTIF($D$233:$D$234, B26)+COUNTIF($D$51:$D$218, B26)+COUNTIF($D$219:$D$220, B26)+COUNTIF($D$1:$D$50, B26)&gt;1,NOT(ISBLANK(B26)))</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="95" priority="1244" stopIfTrue="1">
       <formula>AND(COUNTIF($D$1:$D$191, B26)+COUNTIF($D$214:$D$65380, B26)&gt;1,NOT(ISBLANK(B26)))</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="95" priority="1247" stopIfTrue="1">
-      <formula>AND(COUNTIF($D$474:$D$65380, B26)+COUNTIF($D$454:$D$455, B26)+COUNTIF($D$416:$D$417, B26)+COUNTIF($D$374:$D$377, B26)+COUNTIF($D$351:$D$352, B26)+COUNTIF($D$324:$D$325, B26)+COUNTIF($D$303:$D$303, B26)+COUNTIF($D$288:$D$289, B26)+COUNTIF($D$263:$D$263, B26)+COUNTIF($D$252:$D$253, B26)+COUNTIF($D$233:$D$234, B26)+COUNTIF($D$51:$D$218, B26)+COUNTIF($D$219:$D$220, B26)+COUNTIF($D$1:$D$50, B26)&gt;1,NOT(ISBLANK(B26)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B27">
@@ -4726,55 +4726,55 @@
     <cfRule type="duplicateValues" dxfId="88" priority="347"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="L4">
-    <cfRule type="expression" dxfId="87" priority="1220" stopIfTrue="1">
+    <cfRule type="expression" dxfId="87" priority="1221" stopIfTrue="1">
+      <formula>AND(COUNTIF($C$1:$C$65460, L4)+COUNTIF(#REF!, L4)&gt;1,NOT(ISBLANK(L4)))</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="86" priority="1220" stopIfTrue="1">
       <formula>AND(COUNTIF($C$314:$C$65460, L4)+COUNTIF($C$294:$C$295, L4)+COUNTIF($C$256:$C$257, L4)+COUNTIF($C$214:$C$217, L4)+COUNTIF($C$191:$C$192, L4)+COUNTIF($C$164:$C$165, L4)+COUNTIF($C$143:$C$143, L4)+COUNTIF($C$128:$C$129, L4)+COUNTIF($C$103:$C$103, L4)+COUNTIF($C$92:$C$93, L4)+COUNTIF($C$73:$C$74, L4)+COUNTIF($C$29:$C$56, L4)+COUNTIF($C$58:$C$60, L4)+COUNTIF($C$1:$C$27, L4)&gt;1,NOT(ISBLANK(L4)))</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="86" priority="1221" stopIfTrue="1">
-      <formula>AND(COUNTIF($C$1:$C$65460, L4)+COUNTIF(#REF!, L4)&gt;1,NOT(ISBLANK(L4)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M4">
-    <cfRule type="expression" dxfId="85" priority="1222" stopIfTrue="1">
+    <cfRule type="expression" dxfId="85" priority="1223" stopIfTrue="1">
+      <formula>AND(COUNTIF($D$314:$D$65460, M4)+COUNTIF(#REF!, M4)+COUNTIF($D$1:$D$27, M4)+COUNTIF($D$294:$D$295, M4)+COUNTIF($D$256:$D$257, M4)+COUNTIF($D$214:$D$217, M4)+COUNTIF($D$191:$D$192, M4)+COUNTIF($D$164:$D$165, M4)+COUNTIF($D$143:$D$143, M4)+COUNTIF($D$128:$D$129, M4)+COUNTIF($D$103:$D$103, M4)+COUNTIF($D$92:$D$93, M4)+COUNTIF($D$73:$D$74, M4)+COUNTIF($D$58:$D$60, M4)&gt;1,NOT(ISBLANK(M4)))</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="84" priority="1224" stopIfTrue="1">
+      <formula>AND(COUNTIF($D$294:$D$65460, M4)+COUNTIF($D$1:$D$27, M4)+COUNTIF($D$256:$D$257, M4)+COUNTIF(#REF!, M4)+COUNTIF($D$214:$D$217, M4)+COUNTIF($D$191:$D$192, M4)+COUNTIF($D$164:$D$165, M4)+COUNTIF($D$143:$D$143, M4)+COUNTIF($D$128:$D$129, M4)+COUNTIF($D$103:$D$103, M4)+COUNTIF($D$92:$D$93, M4)+COUNTIF($D$73:$D$74, M4)+COUNTIF($D$58:$D$60, M4)&gt;1,NOT(ISBLANK(M4)))</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="83" priority="1225" stopIfTrue="1">
+      <formula>AND(COUNTIF($D$256:$D$65460, M4)+COUNTIF($D$1:$D$27, M4)+COUNTIF(#REF!, M4)+COUNTIF($D$214:$D$217, M4)+COUNTIF($D$191:$D$192, M4)+COUNTIF($D$164:$D$165, M4)+COUNTIF($D$143:$D$143, M4)+COUNTIF($D$128:$D$129, M4)+COUNTIF($D$103:$D$103, M4)+COUNTIF($D$92:$D$93, M4)+COUNTIF($D$73:$D$74, M4)+COUNTIF($D$58:$D$60, M4)&gt;1,NOT(ISBLANK(M4)))</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="82" priority="1226" stopIfTrue="1">
+      <formula>AND(COUNTIF($D$214:$D$65460, M4)+COUNTIF(#REF!, M4)+COUNTIF($D$1:$D$27, M4)+COUNTIF($D$191:$D$192, M4)+COUNTIF($D$164:$D$165, M4)+COUNTIF($D$143:$D$143, M4)+COUNTIF($D$128:$D$129, M4)+COUNTIF($D$103:$D$103, M4)+COUNTIF($D$92:$D$93, M4)+COUNTIF($D$73:$D$74, M4)+COUNTIF($D$58:$D$60, M4)&gt;1,NOT(ISBLANK(M4)))</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="81" priority="1227" stopIfTrue="1">
+      <formula>AND(COUNTIF($D$214:$D$65460, M4)+COUNTIF($D$191:$D$192, M4)+COUNTIF($D$164:$D$165, M4)+COUNTIF($D$143:$D$143, M4)+COUNTIF($D$128:$D$129, M4)+COUNTIF($D$1:$D$27, M4)+COUNTIF(#REF!, M4)+COUNTIF($D$103:$D$103, M4)+COUNTIF($D$92:$D$93, M4)+COUNTIF(#REF!, M4)+COUNTIF($D$73:$D$74, M4)+COUNTIF($D$51:$D$51, M4)+COUNTIF($D$53:$D$60, M4)+COUNTIF(#REF!, M4)&gt;1,NOT(ISBLANK(M4)))</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="80" priority="1228" stopIfTrue="1">
+      <formula>AND(COUNTIF($D$191:$D$65460, M4)+COUNTIF($D$164:$D$165, M4)+COUNTIF($D$143:$D$143, M4)+COUNTIF($D$128:$D$129, M4)+COUNTIF($D$1:$D$27, M4)+COUNTIF(#REF!, M4)+COUNTIF($D$103:$D$103, M4)+COUNTIF($D$92:$D$93, M4)+COUNTIF(#REF!, M4)+COUNTIF($D$73:$D$74, M4)+COUNTIF($D$51:$D$51, M4)+COUNTIF($D$53:$D$60, M4)+COUNTIF(#REF!, M4)&gt;1,NOT(ISBLANK(M4)))</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="79" priority="1229" stopIfTrue="1">
+      <formula>AND(COUNTIF($F$369:$F$65454, M4)+COUNTIF($F$1:$F$27, M4)+COUNTIF(#REF!, M4)+COUNTIF($F$352:$F$353, M4)+COUNTIF($F$332:$F$333, M4)+COUNTIF($F$294:$F$295, M4)+COUNTIF($F$252:$F$255, M4)+COUNTIF($F$229:$F$230, M4)+COUNTIF($F$202:$F$203, M4)+COUNTIF($F$181:$F$181, M4)+COUNTIF($F$166:$F$167, M4)+COUNTIF($F$141:$F$141, M4)+COUNTIF($F$130:$F$131, M4)+COUNTIF($F$111:$F$112, M4)+COUNTIF($F$96:$F$98, M4)&gt;1,NOT(ISBLANK(M4)))</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="78" priority="1230" stopIfTrue="1">
+      <formula>AND(COUNTIF($F$352:$F$65454, M4)+COUNTIF(#REF!, M4)+COUNTIF($F$1:$F$27, M4)+COUNTIF($F$332:$F$333, M4)+COUNTIF($F$294:$F$295, M4)+COUNTIF($F$252:$F$255, M4)+COUNTIF($F$229:$F$230, M4)+COUNTIF($F$202:$F$203, M4)+COUNTIF($F$181:$F$181, M4)+COUNTIF($F$166:$F$167, M4)+COUNTIF($F$141:$F$141, M4)+COUNTIF($F$130:$F$131, M4)+COUNTIF($F$111:$F$112, M4)+COUNTIF($F$96:$F$98, M4)&gt;1,NOT(ISBLANK(M4)))</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="77" priority="1231" stopIfTrue="1">
+      <formula>AND(COUNTIF($F$332:$F$65454, M4)+COUNTIF($F$1:$F$27, M4)+COUNTIF($F$294:$F$295, M4)+COUNTIF(#REF!, M4)+COUNTIF($F$252:$F$255, M4)+COUNTIF($F$229:$F$230, M4)+COUNTIF($F$202:$F$203, M4)+COUNTIF($F$181:$F$181, M4)+COUNTIF($F$166:$F$167, M4)+COUNTIF($F$141:$F$141, M4)+COUNTIF($F$130:$F$131, M4)+COUNTIF($F$111:$F$112, M4)+COUNTIF($F$96:$F$98, M4)&gt;1,NOT(ISBLANK(M4)))</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="76" priority="1232" stopIfTrue="1">
+      <formula>AND(COUNTIF($F$294:$F$65454, M4)+COUNTIF($F$1:$F$27, M4)+COUNTIF(#REF!, M4)+COUNTIF($F$252:$F$255, M4)+COUNTIF($F$229:$F$230, M4)+COUNTIF($F$202:$F$203, M4)+COUNTIF($F$181:$F$181, M4)+COUNTIF($F$166:$F$167, M4)+COUNTIF($F$141:$F$141, M4)+COUNTIF($F$130:$F$131, M4)+COUNTIF($F$111:$F$112, M4)+COUNTIF($F$96:$F$98, M4)&gt;1,NOT(ISBLANK(M4)))</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="75" priority="1233" stopIfTrue="1">
+      <formula>AND(COUNTIF($F$252:$F$65454, M4)+COUNTIF(#REF!, M4)+COUNTIF($F$1:$F$27, M4)+COUNTIF($F$229:$F$230, M4)+COUNTIF($F$202:$F$203, M4)+COUNTIF($F$181:$F$181, M4)+COUNTIF($F$166:$F$167, M4)+COUNTIF($F$141:$F$141, M4)+COUNTIF($F$130:$F$131, M4)+COUNTIF($F$111:$F$112, M4)+COUNTIF($F$96:$F$98, M4)&gt;1,NOT(ISBLANK(M4)))</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="74" priority="1234" stopIfTrue="1">
+      <formula>AND(COUNTIF($F$252:$F$65454, M4)+COUNTIF($F$229:$F$230, M4)+COUNTIF($F$202:$F$203, M4)+COUNTIF($F$181:$F$181, M4)+COUNTIF($F$166:$F$167, M4)+COUNTIF($F$1:$F$27, M4)+COUNTIF(#REF!, M4)+COUNTIF($F$141:$F$141, M4)+COUNTIF($F$130:$F$131, M4)+COUNTIF(#REF!, M4)+COUNTIF($F$111:$F$112, M4)+COUNTIF($F$89:$F$89, M4)+COUNTIF($F$91:$F$98, M4)+COUNTIF(#REF!, M4)&gt;1,NOT(ISBLANK(M4)))</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="73" priority="1235" stopIfTrue="1">
+      <formula>AND(COUNTIF($F$229:$F$65454, M4)+COUNTIF($F$202:$F$203, M4)+COUNTIF($F$181:$F$181, M4)+COUNTIF($F$166:$F$167, M4)+COUNTIF($F$1:$F$27, M4)+COUNTIF(#REF!, M4)+COUNTIF($F$141:$F$141, M4)+COUNTIF($F$130:$F$131, M4)+COUNTIF(#REF!, M4)+COUNTIF($F$111:$F$112, M4)+COUNTIF($F$89:$F$89, M4)+COUNTIF($F$91:$F$98, M4)+COUNTIF(#REF!, M4)&gt;1,NOT(ISBLANK(M4)))</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="72" priority="1222" stopIfTrue="1">
       <formula>AND(COUNTIF($D$331:$D$65460, M4)+COUNTIF($D$1:$D$27, M4)+COUNTIF(#REF!, M4)+COUNTIF($D$314:$D$315, M4)+COUNTIF($D$294:$D$295, M4)+COUNTIF($D$256:$D$257, M4)+COUNTIF($D$214:$D$217, M4)+COUNTIF($D$191:$D$192, M4)+COUNTIF($D$164:$D$165, M4)+COUNTIF($D$143:$D$143, M4)+COUNTIF($D$128:$D$129, M4)+COUNTIF($D$103:$D$103, M4)+COUNTIF($D$92:$D$93, M4)+COUNTIF($D$73:$D$74, M4)+COUNTIF($D$58:$D$60, M4)&gt;1,NOT(ISBLANK(M4)))</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="84" priority="1223" stopIfTrue="1">
-      <formula>AND(COUNTIF($D$314:$D$65460, M4)+COUNTIF(#REF!, M4)+COUNTIF($D$1:$D$27, M4)+COUNTIF($D$294:$D$295, M4)+COUNTIF($D$256:$D$257, M4)+COUNTIF($D$214:$D$217, M4)+COUNTIF($D$191:$D$192, M4)+COUNTIF($D$164:$D$165, M4)+COUNTIF($D$143:$D$143, M4)+COUNTIF($D$128:$D$129, M4)+COUNTIF($D$103:$D$103, M4)+COUNTIF($D$92:$D$93, M4)+COUNTIF($D$73:$D$74, M4)+COUNTIF($D$58:$D$60, M4)&gt;1,NOT(ISBLANK(M4)))</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="83" priority="1224" stopIfTrue="1">
-      <formula>AND(COUNTIF($D$294:$D$65460, M4)+COUNTIF($D$1:$D$27, M4)+COUNTIF($D$256:$D$257, M4)+COUNTIF(#REF!, M4)+COUNTIF($D$214:$D$217, M4)+COUNTIF($D$191:$D$192, M4)+COUNTIF($D$164:$D$165, M4)+COUNTIF($D$143:$D$143, M4)+COUNTIF($D$128:$D$129, M4)+COUNTIF($D$103:$D$103, M4)+COUNTIF($D$92:$D$93, M4)+COUNTIF($D$73:$D$74, M4)+COUNTIF($D$58:$D$60, M4)&gt;1,NOT(ISBLANK(M4)))</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="82" priority="1225" stopIfTrue="1">
-      <formula>AND(COUNTIF($D$256:$D$65460, M4)+COUNTIF($D$1:$D$27, M4)+COUNTIF(#REF!, M4)+COUNTIF($D$214:$D$217, M4)+COUNTIF($D$191:$D$192, M4)+COUNTIF($D$164:$D$165, M4)+COUNTIF($D$143:$D$143, M4)+COUNTIF($D$128:$D$129, M4)+COUNTIF($D$103:$D$103, M4)+COUNTIF($D$92:$D$93, M4)+COUNTIF($D$73:$D$74, M4)+COUNTIF($D$58:$D$60, M4)&gt;1,NOT(ISBLANK(M4)))</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="81" priority="1226" stopIfTrue="1">
-      <formula>AND(COUNTIF($D$214:$D$65460, M4)+COUNTIF(#REF!, M4)+COUNTIF($D$1:$D$27, M4)+COUNTIF($D$191:$D$192, M4)+COUNTIF($D$164:$D$165, M4)+COUNTIF($D$143:$D$143, M4)+COUNTIF($D$128:$D$129, M4)+COUNTIF($D$103:$D$103, M4)+COUNTIF($D$92:$D$93, M4)+COUNTIF($D$73:$D$74, M4)+COUNTIF($D$58:$D$60, M4)&gt;1,NOT(ISBLANK(M4)))</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="80" priority="1227" stopIfTrue="1">
-      <formula>AND(COUNTIF($D$214:$D$65460, M4)+COUNTIF($D$191:$D$192, M4)+COUNTIF($D$164:$D$165, M4)+COUNTIF($D$143:$D$143, M4)+COUNTIF($D$128:$D$129, M4)+COUNTIF($D$1:$D$27, M4)+COUNTIF(#REF!, M4)+COUNTIF($D$103:$D$103, M4)+COUNTIF($D$92:$D$93, M4)+COUNTIF(#REF!, M4)+COUNTIF($D$73:$D$74, M4)+COUNTIF($D$51:$D$51, M4)+COUNTIF($D$53:$D$60, M4)+COUNTIF(#REF!, M4)&gt;1,NOT(ISBLANK(M4)))</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="79" priority="1228" stopIfTrue="1">
-      <formula>AND(COUNTIF($D$191:$D$65460, M4)+COUNTIF($D$164:$D$165, M4)+COUNTIF($D$143:$D$143, M4)+COUNTIF($D$128:$D$129, M4)+COUNTIF($D$1:$D$27, M4)+COUNTIF(#REF!, M4)+COUNTIF($D$103:$D$103, M4)+COUNTIF($D$92:$D$93, M4)+COUNTIF(#REF!, M4)+COUNTIF($D$73:$D$74, M4)+COUNTIF($D$51:$D$51, M4)+COUNTIF($D$53:$D$60, M4)+COUNTIF(#REF!, M4)&gt;1,NOT(ISBLANK(M4)))</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="78" priority="1229" stopIfTrue="1">
-      <formula>AND(COUNTIF($F$369:$F$65454, M4)+COUNTIF($F$1:$F$27, M4)+COUNTIF(#REF!, M4)+COUNTIF($F$352:$F$353, M4)+COUNTIF($F$332:$F$333, M4)+COUNTIF($F$294:$F$295, M4)+COUNTIF($F$252:$F$255, M4)+COUNTIF($F$229:$F$230, M4)+COUNTIF($F$202:$F$203, M4)+COUNTIF($F$181:$F$181, M4)+COUNTIF($F$166:$F$167, M4)+COUNTIF($F$141:$F$141, M4)+COUNTIF($F$130:$F$131, M4)+COUNTIF($F$111:$F$112, M4)+COUNTIF($F$96:$F$98, M4)&gt;1,NOT(ISBLANK(M4)))</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="77" priority="1230" stopIfTrue="1">
-      <formula>AND(COUNTIF($F$352:$F$65454, M4)+COUNTIF(#REF!, M4)+COUNTIF($F$1:$F$27, M4)+COUNTIF($F$332:$F$333, M4)+COUNTIF($F$294:$F$295, M4)+COUNTIF($F$252:$F$255, M4)+COUNTIF($F$229:$F$230, M4)+COUNTIF($F$202:$F$203, M4)+COUNTIF($F$181:$F$181, M4)+COUNTIF($F$166:$F$167, M4)+COUNTIF($F$141:$F$141, M4)+COUNTIF($F$130:$F$131, M4)+COUNTIF($F$111:$F$112, M4)+COUNTIF($F$96:$F$98, M4)&gt;1,NOT(ISBLANK(M4)))</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="76" priority="1231" stopIfTrue="1">
-      <formula>AND(COUNTIF($F$332:$F$65454, M4)+COUNTIF($F$1:$F$27, M4)+COUNTIF($F$294:$F$295, M4)+COUNTIF(#REF!, M4)+COUNTIF($F$252:$F$255, M4)+COUNTIF($F$229:$F$230, M4)+COUNTIF($F$202:$F$203, M4)+COUNTIF($F$181:$F$181, M4)+COUNTIF($F$166:$F$167, M4)+COUNTIF($F$141:$F$141, M4)+COUNTIF($F$130:$F$131, M4)+COUNTIF($F$111:$F$112, M4)+COUNTIF($F$96:$F$98, M4)&gt;1,NOT(ISBLANK(M4)))</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="75" priority="1232" stopIfTrue="1">
-      <formula>AND(COUNTIF($F$294:$F$65454, M4)+COUNTIF($F$1:$F$27, M4)+COUNTIF(#REF!, M4)+COUNTIF($F$252:$F$255, M4)+COUNTIF($F$229:$F$230, M4)+COUNTIF($F$202:$F$203, M4)+COUNTIF($F$181:$F$181, M4)+COUNTIF($F$166:$F$167, M4)+COUNTIF($F$141:$F$141, M4)+COUNTIF($F$130:$F$131, M4)+COUNTIF($F$111:$F$112, M4)+COUNTIF($F$96:$F$98, M4)&gt;1,NOT(ISBLANK(M4)))</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="74" priority="1233" stopIfTrue="1">
-      <formula>AND(COUNTIF($F$252:$F$65454, M4)+COUNTIF(#REF!, M4)+COUNTIF($F$1:$F$27, M4)+COUNTIF($F$229:$F$230, M4)+COUNTIF($F$202:$F$203, M4)+COUNTIF($F$181:$F$181, M4)+COUNTIF($F$166:$F$167, M4)+COUNTIF($F$141:$F$141, M4)+COUNTIF($F$130:$F$131, M4)+COUNTIF($F$111:$F$112, M4)+COUNTIF($F$96:$F$98, M4)&gt;1,NOT(ISBLANK(M4)))</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="73" priority="1234" stopIfTrue="1">
-      <formula>AND(COUNTIF($F$252:$F$65454, M4)+COUNTIF($F$229:$F$230, M4)+COUNTIF($F$202:$F$203, M4)+COUNTIF($F$181:$F$181, M4)+COUNTIF($F$166:$F$167, M4)+COUNTIF($F$1:$F$27, M4)+COUNTIF(#REF!, M4)+COUNTIF($F$141:$F$141, M4)+COUNTIF($F$130:$F$131, M4)+COUNTIF(#REF!, M4)+COUNTIF($F$111:$F$112, M4)+COUNTIF($F$89:$F$89, M4)+COUNTIF($F$91:$F$98, M4)+COUNTIF(#REF!, M4)&gt;1,NOT(ISBLANK(M4)))</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="72" priority="1235" stopIfTrue="1">
-      <formula>AND(COUNTIF($F$229:$F$65454, M4)+COUNTIF($F$202:$F$203, M4)+COUNTIF($F$181:$F$181, M4)+COUNTIF($F$166:$F$167, M4)+COUNTIF($F$1:$F$27, M4)+COUNTIF(#REF!, M4)+COUNTIF($F$141:$F$141, M4)+COUNTIF($F$130:$F$131, M4)+COUNTIF(#REF!, M4)+COUNTIF($F$111:$F$112, M4)+COUNTIF($F$89:$F$89, M4)+COUNTIF($F$91:$F$98, M4)+COUNTIF(#REF!, M4)&gt;1,NOT(ISBLANK(M4)))</formula>
     </cfRule>
   </conditionalFormatting>
   <printOptions horizontalCentered="1"/>
@@ -5135,7 +5135,9 @@
       <c r="E3" s="138" t="s">
         <v>179</v>
       </c>
-      <c r="F3" s="141"/>
+      <c r="F3" s="139">
+        <v>27</v>
+      </c>
       <c r="G3" s="138" t="s">
         <v>167</v>
       </c>
@@ -5200,7 +5202,9 @@
       <c r="E4" s="138" t="s">
         <v>179</v>
       </c>
-      <c r="F4" s="138"/>
+      <c r="F4" s="139">
+        <v>27</v>
+      </c>
       <c r="G4" s="138" t="s">
         <v>167</v>
       </c>
@@ -5265,7 +5269,9 @@
       <c r="E5" s="138" t="s">
         <v>179</v>
       </c>
-      <c r="F5" s="141"/>
+      <c r="F5" s="139">
+        <v>27</v>
+      </c>
       <c r="G5" s="138" t="s">
         <v>167</v>
       </c>
@@ -5330,7 +5336,9 @@
       <c r="E6" s="138" t="s">
         <v>179</v>
       </c>
-      <c r="F6" s="138"/>
+      <c r="F6" s="139">
+        <v>27</v>
+      </c>
       <c r="G6" s="138" t="s">
         <v>167</v>
       </c>
@@ -5395,7 +5403,9 @@
       <c r="E7" s="138" t="s">
         <v>179</v>
       </c>
-      <c r="F7" s="141"/>
+      <c r="F7" s="139">
+        <v>27</v>
+      </c>
       <c r="G7" s="138" t="s">
         <v>167</v>
       </c>
@@ -5515,7 +5525,9 @@
       <c r="E9" s="138" t="s">
         <v>161</v>
       </c>
-      <c r="F9" s="141"/>
+      <c r="F9" s="139">
+        <v>35</v>
+      </c>
       <c r="G9" s="138" t="s">
         <v>167</v>
       </c>
@@ -5579,7 +5591,9 @@
       <c r="E10" s="138" t="s">
         <v>161</v>
       </c>
-      <c r="F10" s="141"/>
+      <c r="F10" s="139">
+        <v>35</v>
+      </c>
       <c r="G10" s="138" t="s">
         <v>167</v>
       </c>
@@ -5644,7 +5658,9 @@
       <c r="E11" s="138" t="s">
         <v>161</v>
       </c>
-      <c r="F11" s="141"/>
+      <c r="F11" s="139">
+        <v>35</v>
+      </c>
       <c r="G11" s="138" t="s">
         <v>167</v>
       </c>
@@ -5709,7 +5725,9 @@
       <c r="E12" s="138" t="s">
         <v>161</v>
       </c>
-      <c r="F12" s="135"/>
+      <c r="F12" s="139">
+        <v>35</v>
+      </c>
       <c r="G12" s="138" t="s">
         <v>167</v>
       </c>
@@ -5774,7 +5792,9 @@
       <c r="E13" s="138" t="s">
         <v>161</v>
       </c>
-      <c r="F13" s="135"/>
+      <c r="F13" s="139">
+        <v>35</v>
+      </c>
       <c r="G13" s="138" t="s">
         <v>167</v>
       </c>
@@ -5839,7 +5859,9 @@
       <c r="E14" s="138" t="s">
         <v>161</v>
       </c>
-      <c r="F14" s="141"/>
+      <c r="F14" s="139">
+        <v>35</v>
+      </c>
       <c r="G14" s="138" t="s">
         <v>167</v>
       </c>
@@ -5960,7 +5982,9 @@
       <c r="E16" s="138" t="s">
         <v>162</v>
       </c>
-      <c r="F16" s="135"/>
+      <c r="F16" s="139">
+        <v>30</v>
+      </c>
       <c r="G16" s="138" t="s">
         <v>168</v>
       </c>
@@ -6025,7 +6049,9 @@
       <c r="E17" s="138" t="s">
         <v>162</v>
       </c>
-      <c r="F17" s="135"/>
+      <c r="F17" s="139">
+        <v>30</v>
+      </c>
       <c r="G17" s="138" t="s">
         <v>168</v>
       </c>
@@ -6090,7 +6116,9 @@
       <c r="E18" s="138" t="s">
         <v>162</v>
       </c>
-      <c r="F18" s="141"/>
+      <c r="F18" s="139">
+        <v>30</v>
+      </c>
       <c r="G18" s="138" t="s">
         <v>168</v>
       </c>
@@ -6221,7 +6249,9 @@
       <c r="E20" s="138" t="s">
         <v>163</v>
       </c>
-      <c r="F20" s="138"/>
+      <c r="F20" s="139">
+        <v>20</v>
+      </c>
       <c r="G20" s="138" t="s">
         <v>168</v>
       </c>
@@ -6286,7 +6316,9 @@
       <c r="E21" s="138" t="s">
         <v>163</v>
       </c>
-      <c r="F21" s="138"/>
+      <c r="F21" s="139">
+        <v>20</v>
+      </c>
       <c r="G21" s="138" t="s">
         <v>168</v>
       </c>
@@ -6351,7 +6383,9 @@
       <c r="E22" s="138" t="s">
         <v>163</v>
       </c>
-      <c r="F22" s="141"/>
+      <c r="F22" s="139">
+        <v>20</v>
+      </c>
       <c r="G22" s="138" t="s">
         <v>168</v>
       </c>
@@ -6475,7 +6509,9 @@
       <c r="E24" s="138" t="s">
         <v>164</v>
       </c>
-      <c r="F24" s="141"/>
+      <c r="F24" s="139">
+        <v>20</v>
+      </c>
       <c r="G24" s="138" t="s">
         <v>168</v>
       </c>
@@ -6539,7 +6575,9 @@
       <c r="E25" s="138" t="s">
         <v>164</v>
       </c>
-      <c r="F25" s="141"/>
+      <c r="F25" s="139">
+        <v>20</v>
+      </c>
       <c r="G25" s="138" t="s">
         <v>168</v>
       </c>
@@ -6603,7 +6641,9 @@
       <c r="E26" s="138" t="s">
         <v>164</v>
       </c>
-      <c r="F26" s="141"/>
+      <c r="F26" s="139">
+        <v>20</v>
+      </c>
       <c r="G26" s="138" t="s">
         <v>168</v>
       </c>
@@ -6668,7 +6708,9 @@
       <c r="E27" s="138" t="s">
         <v>164</v>
       </c>
-      <c r="F27" s="141"/>
+      <c r="F27" s="139">
+        <v>20</v>
+      </c>
       <c r="G27" s="138" t="s">
         <v>168</v>
       </c>
@@ -6988,12 +7030,12 @@
     <cfRule type="duplicateValues" dxfId="68" priority="1379"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B17">
-    <cfRule type="duplicateValues" dxfId="67" priority="123"/>
-    <cfRule type="duplicateValues" dxfId="66" priority="124"/>
+    <cfRule type="duplicateValues" dxfId="67" priority="124"/>
+    <cfRule type="duplicateValues" dxfId="66" priority="123"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B18">
-    <cfRule type="duplicateValues" dxfId="65" priority="125"/>
-    <cfRule type="duplicateValues" dxfId="64" priority="126"/>
+    <cfRule type="duplicateValues" dxfId="65" priority="126"/>
+    <cfRule type="duplicateValues" dxfId="64" priority="125"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B26:B27 B2:B3 B21:B23 B5:B19">
     <cfRule type="duplicateValues" dxfId="63" priority="1367"/>
@@ -7005,28 +7047,28 @@
     <cfRule type="duplicateValues" dxfId="61" priority="160"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="J2:J14 K16 J16:J31">
-    <cfRule type="containsText" dxfId="60" priority="179" operator="containsText" text="WIP">
-      <formula>NOT(ISERROR(SEARCH("WIP",J2)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="59" priority="182" operator="containsText" text="Complete">
+    <cfRule type="containsText" dxfId="60" priority="198" operator="containsText" text="ROW">
+      <formula>NOT(ISERROR(SEARCH("ROW",J2)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="59" priority="197" operator="containsText" text="Complete">
       <formula>NOT(ISERROR(SEARCH("Complete",J2)))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="58" priority="183" operator="containsText" text="ROW">
       <formula>NOT(ISERROR(SEARCH("ROW",J2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="57" priority="197" operator="containsText" text="Complete">
+    <cfRule type="containsText" dxfId="57" priority="182" operator="containsText" text="Complete">
       <formula>NOT(ISERROR(SEARCH("Complete",J2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="56" priority="198" operator="containsText" text="ROW">
-      <formula>NOT(ISERROR(SEARCH("ROW",J2)))</formula>
+    <cfRule type="containsText" dxfId="56" priority="179" operator="containsText" text="WIP">
+      <formula>NOT(ISERROR(SEARCH("WIP",J2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K3:K7 K9:K13 K20:K22">
-    <cfRule type="containsText" dxfId="55" priority="111" operator="containsText" text="Complete">
+    <cfRule type="containsText" dxfId="55" priority="112" operator="containsText" text="ROW">
+      <formula>NOT(ISERROR(SEARCH("ROW",K3)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="54" priority="111" operator="containsText" text="Complete">
       <formula>NOT(ISERROR(SEARCH("Complete",K3)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="54" priority="112" operator="containsText" text="ROW">
-      <formula>NOT(ISERROR(SEARCH("ROW",K3)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K3:K7 K9:K13 K20:N22">
@@ -7035,19 +7077,19 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K3:K7 L4:L5 K9:K13">
-    <cfRule type="containsText" dxfId="52" priority="108" operator="containsText" text="Complete">
+    <cfRule type="containsText" dxfId="52" priority="109" operator="containsText" text="ROW">
+      <formula>NOT(ISERROR(SEARCH("ROW",K3)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="51" priority="108" operator="containsText" text="Complete">
       <formula>NOT(ISERROR(SEARCH("Complete",K3)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="51" priority="109" operator="containsText" text="ROW">
-      <formula>NOT(ISERROR(SEARCH("ROW",K3)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K3:K7">
-    <cfRule type="containsText" dxfId="50" priority="70" operator="containsText" text="Complete">
+    <cfRule type="containsText" dxfId="50" priority="71" operator="containsText" text="ROW">
+      <formula>NOT(ISERROR(SEARCH("ROW",K3)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="49" priority="70" operator="containsText" text="Complete">
       <formula>NOT(ISERROR(SEARCH("Complete",K3)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="49" priority="71" operator="containsText" text="ROW">
-      <formula>NOT(ISERROR(SEARCH("ROW",K3)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K16:M16 L2:N7 L9:N14 O24 O26:O30 L8:M8 N15 K17:N18 L23:N26 K25:K26 K27:N31">
@@ -7056,19 +7098,19 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K20:N22">
-    <cfRule type="containsText" dxfId="47" priority="66" operator="containsText" text="Complete">
+    <cfRule type="containsText" dxfId="47" priority="67" operator="containsText" text="ROW">
+      <formula>NOT(ISERROR(SEARCH("ROW",K20)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="46" priority="66" operator="containsText" text="Complete">
       <formula>NOT(ISERROR(SEARCH("Complete",K20)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="46" priority="67" operator="containsText" text="ROW">
-      <formula>NOT(ISERROR(SEARCH("ROW",K20)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L10:L11">
-    <cfRule type="containsText" dxfId="45" priority="72" operator="containsText" text="Complete">
+    <cfRule type="containsText" dxfId="45" priority="73" operator="containsText" text="ROW">
+      <formula>NOT(ISERROR(SEARCH("ROW",L10)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="44" priority="72" operator="containsText" text="Complete">
       <formula>NOT(ISERROR(SEARCH("Complete",L10)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="44" priority="73" operator="containsText" text="ROW">
-      <formula>NOT(ISERROR(SEARCH("ROW",L10)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L15">
@@ -7093,11 +7135,11 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L19:N19">
-    <cfRule type="containsText" dxfId="38" priority="17" operator="containsText" text="Complete">
+    <cfRule type="containsText" dxfId="38" priority="18" operator="containsText" text="ROW">
+      <formula>NOT(ISERROR(SEARCH("ROW",L19)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="37" priority="17" operator="containsText" text="Complete">
       <formula>NOT(ISERROR(SEARCH("Complete",L19)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="37" priority="18" operator="containsText" text="ROW">
-      <formula>NOT(ISERROR(SEARCH("ROW",L19)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L19:O19">
@@ -7146,33 +7188,33 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O9">
-    <cfRule type="containsText" dxfId="25" priority="26" operator="containsText" text="WIP">
-      <formula>NOT(ISERROR(SEARCH("WIP",O9)))</formula>
+    <cfRule type="containsText" dxfId="25" priority="28" operator="containsText" text="ROW">
+      <formula>NOT(ISERROR(SEARCH("ROW",O9)))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="24" priority="27" operator="containsText" text="Complete">
       <formula>NOT(ISERROR(SEARCH("Complete",O9)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="23" priority="28" operator="containsText" text="ROW">
-      <formula>NOT(ISERROR(SEARCH("ROW",O9)))</formula>
+    <cfRule type="containsText" dxfId="23" priority="26" operator="containsText" text="WIP">
+      <formula>NOT(ISERROR(SEARCH("WIP",O9)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O10">
-    <cfRule type="containsText" dxfId="22" priority="57" operator="containsText" text="WIP">
+    <cfRule type="containsText" dxfId="22" priority="58" operator="containsText" text="Complete">
+      <formula>NOT(ISERROR(SEARCH("Complete",O10)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="21" priority="59" operator="containsText" text="ROW">
+      <formula>NOT(ISERROR(SEARCH("ROW",O10)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="20" priority="57" operator="containsText" text="WIP">
       <formula>NOT(ISERROR(SEARCH("WIP",O10)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="21" priority="58" operator="containsText" text="Complete">
-      <formula>NOT(ISERROR(SEARCH("Complete",O10)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="20" priority="59" operator="containsText" text="ROW">
-      <formula>NOT(ISERROR(SEARCH("ROW",O10)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O10:O13">
-    <cfRule type="containsText" dxfId="19" priority="55" operator="containsText" text="Complete">
+    <cfRule type="containsText" dxfId="19" priority="56" operator="containsText" text="ROW">
+      <formula>NOT(ISERROR(SEARCH("ROW",O10)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="18" priority="55" operator="containsText" text="Complete">
       <formula>NOT(ISERROR(SEARCH("Complete",O10)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="18" priority="56" operator="containsText" text="ROW">
-      <formula>NOT(ISERROR(SEARCH("ROW",O10)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O11:O13">
@@ -7181,19 +7223,19 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O13">
-    <cfRule type="containsText" dxfId="16" priority="24" operator="containsText" text="Complete">
+    <cfRule type="containsText" dxfId="16" priority="25" operator="containsText" text="ROW">
+      <formula>NOT(ISERROR(SEARCH("ROW",O13)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="15" priority="24" operator="containsText" text="Complete">
       <formula>NOT(ISERROR(SEARCH("Complete",O13)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="15" priority="25" operator="containsText" text="ROW">
-      <formula>NOT(ISERROR(SEARCH("ROW",O13)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O13:O14">
-    <cfRule type="containsText" dxfId="14" priority="52" operator="containsText" text="Complete">
+    <cfRule type="containsText" dxfId="14" priority="53" operator="containsText" text="ROW">
+      <formula>NOT(ISERROR(SEARCH("ROW",O13)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="13" priority="52" operator="containsText" text="Complete">
       <formula>NOT(ISERROR(SEARCH("Complete",O13)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="13" priority="53" operator="containsText" text="ROW">
-      <formula>NOT(ISERROR(SEARCH("ROW",O13)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O13:O17">
@@ -7202,38 +7244,38 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O15:O16">
-    <cfRule type="containsText" dxfId="11" priority="9" operator="containsText" text="Complete">
+    <cfRule type="containsText" dxfId="11" priority="10" operator="containsText" text="ROW">
+      <formula>NOT(ISERROR(SEARCH("ROW",O15)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="10" priority="9" operator="containsText" text="Complete">
       <formula>NOT(ISERROR(SEARCH("Complete",O15)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="10" priority="10" operator="containsText" text="ROW">
-      <formula>NOT(ISERROR(SEARCH("ROW",O15)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O15:O17">
-    <cfRule type="containsText" dxfId="9" priority="12" operator="containsText" text="Complete">
+    <cfRule type="containsText" dxfId="9" priority="13" operator="containsText" text="ROW">
+      <formula>NOT(ISERROR(SEARCH("ROW",O15)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="8" priority="12" operator="containsText" text="Complete">
       <formula>NOT(ISERROR(SEARCH("Complete",O15)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="8" priority="13" operator="containsText" text="ROW">
-      <formula>NOT(ISERROR(SEARCH("ROW",O15)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O19:O20">
-    <cfRule type="containsText" dxfId="7" priority="20" operator="containsText" text="Complete">
+    <cfRule type="containsText" dxfId="7" priority="21" operator="containsText" text="ROW">
+      <formula>NOT(ISERROR(SEARCH("ROW",O19)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="6" priority="20" operator="containsText" text="Complete">
       <formula>NOT(ISERROR(SEARCH("Complete",O19)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="6" priority="21" operator="containsText" text="ROW">
-      <formula>NOT(ISERROR(SEARCH("ROW",O19)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O20:O24">
-    <cfRule type="containsText" dxfId="5" priority="41" operator="containsText" text="WIP">
+    <cfRule type="containsText" dxfId="5" priority="42" operator="containsText" text="Complete">
+      <formula>NOT(ISERROR(SEARCH("Complete",O20)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="4" priority="43" operator="containsText" text="ROW">
+      <formula>NOT(ISERROR(SEARCH("ROW",O20)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="3" priority="41" operator="containsText" text="WIP">
       <formula>NOT(ISERROR(SEARCH("WIP",O20)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="4" priority="42" operator="containsText" text="Complete">
-      <formula>NOT(ISERROR(SEARCH("Complete",O20)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="3" priority="43" operator="containsText" text="ROW">
-      <formula>NOT(ISERROR(SEARCH("ROW",O20)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O26">
@@ -8018,32 +8060,32 @@
       <c r="F17" s="6"/>
     </row>
     <row r="18" spans="1:28" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="180" t="s">
+      <c r="A18" s="195" t="s">
         <v>4</v>
       </c>
-      <c r="B18" s="180" t="s">
+      <c r="B18" s="195" t="s">
         <v>42</v>
       </c>
-      <c r="C18" s="177" t="s">
+      <c r="C18" s="191" t="s">
         <v>47</v>
       </c>
-      <c r="D18" s="177" t="s">
+      <c r="D18" s="191" t="s">
         <v>43</v>
       </c>
-      <c r="E18" s="180" t="s">
+      <c r="E18" s="195" t="s">
         <v>8</v>
       </c>
-      <c r="F18" s="192" t="s">
+      <c r="F18" s="182" t="s">
         <v>18</v>
       </c>
-      <c r="G18" s="192"/>
-      <c r="H18" s="192"/>
-      <c r="I18" s="192"/>
-      <c r="J18" s="192"/>
+      <c r="G18" s="182"/>
+      <c r="H18" s="182"/>
+      <c r="I18" s="182"/>
+      <c r="J18" s="182"/>
       <c r="K18" s="185" t="s">
         <v>19</v>
       </c>
-      <c r="M18" s="177" t="s">
+      <c r="M18" s="191" t="s">
         <v>36</v>
       </c>
       <c r="O18" s="186" t="s">
@@ -8067,24 +8109,24 @@
       </c>
     </row>
     <row r="19" spans="1:28" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="181"/>
-      <c r="B19" s="181"/>
-      <c r="C19" s="178"/>
-      <c r="D19" s="181"/>
-      <c r="E19" s="181"/>
-      <c r="F19" s="204" t="s">
+      <c r="A19" s="196"/>
+      <c r="B19" s="196"/>
+      <c r="C19" s="193"/>
+      <c r="D19" s="196"/>
+      <c r="E19" s="196"/>
+      <c r="F19" s="203" t="s">
         <v>40</v>
       </c>
-      <c r="G19" s="205" t="s">
+      <c r="G19" s="204" t="s">
         <v>44</v>
       </c>
-      <c r="H19" s="206"/>
-      <c r="I19" s="205" t="s">
+      <c r="H19" s="205"/>
+      <c r="I19" s="204" t="s">
         <v>45</v>
       </c>
-      <c r="J19" s="206"/>
+      <c r="J19" s="205"/>
       <c r="K19" s="185"/>
-      <c r="M19" s="191"/>
+      <c r="M19" s="192"/>
       <c r="O19" s="183" t="s">
         <v>24</v>
       </c>
@@ -8124,12 +8166,12 @@
       <c r="AB19" s="190"/>
     </row>
     <row r="20" spans="1:28" ht="36.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A20" s="181"/>
-      <c r="B20" s="181"/>
-      <c r="C20" s="178"/>
-      <c r="D20" s="181"/>
-      <c r="E20" s="181"/>
-      <c r="F20" s="204"/>
+      <c r="A20" s="196"/>
+      <c r="B20" s="196"/>
+      <c r="C20" s="193"/>
+      <c r="D20" s="196"/>
+      <c r="E20" s="196"/>
+      <c r="F20" s="203"/>
       <c r="G20" s="94" t="s">
         <v>10</v>
       </c>
@@ -8179,7 +8221,7 @@
       <c r="D21" s="8" t="s">
         <v>79</v>
       </c>
-      <c r="E21" s="203" t="s">
+      <c r="E21" s="206" t="s">
         <v>98</v>
       </c>
       <c r="F21" s="114">
@@ -8253,7 +8295,7 @@
       <c r="D22" s="8" t="s">
         <v>79</v>
       </c>
-      <c r="E22" s="203"/>
+      <c r="E22" s="206"/>
       <c r="F22" s="114">
         <v>45913</v>
       </c>
@@ -8325,7 +8367,7 @@
       <c r="D23" s="8" t="s">
         <v>86</v>
       </c>
-      <c r="E23" s="203"/>
+      <c r="E23" s="206"/>
       <c r="F23" s="114">
         <v>45910</v>
       </c>
@@ -8397,7 +8439,7 @@
       <c r="D24" s="8" t="s">
         <v>86</v>
       </c>
-      <c r="E24" s="203"/>
+      <c r="E24" s="206"/>
       <c r="F24" s="114">
         <v>45927</v>
       </c>
@@ -8469,7 +8511,7 @@
       <c r="D25" s="8" t="s">
         <v>86</v>
       </c>
-      <c r="E25" s="203"/>
+      <c r="E25" s="206"/>
       <c r="F25" s="114">
         <v>45915</v>
       </c>
@@ -9164,6 +9206,18 @@
     </row>
   </sheetData>
   <mergeCells count="25">
+    <mergeCell ref="E21:E25"/>
+    <mergeCell ref="W19:W20"/>
+    <mergeCell ref="K18:K19"/>
+    <mergeCell ref="M18:M19"/>
+    <mergeCell ref="O18:T18"/>
+    <mergeCell ref="V18:AA18"/>
+    <mergeCell ref="V19:V20"/>
+    <mergeCell ref="A18:A20"/>
+    <mergeCell ref="B18:B20"/>
+    <mergeCell ref="C18:C20"/>
+    <mergeCell ref="D18:D20"/>
+    <mergeCell ref="E18:E20"/>
     <mergeCell ref="AB18:AB19"/>
     <mergeCell ref="F19:F20"/>
     <mergeCell ref="G19:H19"/>
@@ -9177,18 +9231,6 @@
     <mergeCell ref="Q19:Q20"/>
     <mergeCell ref="R19:R20"/>
     <mergeCell ref="S19:S20"/>
-    <mergeCell ref="A18:A20"/>
-    <mergeCell ref="B18:B20"/>
-    <mergeCell ref="C18:C20"/>
-    <mergeCell ref="D18:D20"/>
-    <mergeCell ref="E18:E20"/>
-    <mergeCell ref="E21:E25"/>
-    <mergeCell ref="W19:W20"/>
-    <mergeCell ref="K18:K19"/>
-    <mergeCell ref="M18:M19"/>
-    <mergeCell ref="O18:T18"/>
-    <mergeCell ref="V18:AA18"/>
-    <mergeCell ref="V19:V20"/>
   </mergeCells>
   <conditionalFormatting sqref="C26:C27">
     <cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="4DT6">

</xml_diff>